<commit_message>
csv reader, about to delete hardcoded equipment templates
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="194">
   <si>
     <t>baseItem</t>
   </si>
@@ -508,16 +508,10 @@
     <t>Suffix:PercentArmorClass</t>
   </si>
   <si>
-    <t>affixCategory</t>
-  </si>
-  <si>
     <t>affixType</t>
   </si>
   <si>
     <t>maxTier</t>
-  </si>
-  <si>
-    <t>Suffix</t>
   </si>
   <si>
     <t>FlatDamage</t>
@@ -2508,48 +2502,48 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B2">
         <v>7</v>
@@ -2578,7 +2572,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -2601,7 +2595,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D4">
         <v>14</v>
@@ -2618,7 +2612,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -2635,7 +2629,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -2643,7 +2637,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B7">
         <v>8</v>
@@ -2672,7 +2666,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B8">
         <v>3</v>
@@ -2704,7 +2698,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B9">
         <v>5</v>
@@ -2733,7 +2727,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B10">
         <v>4</v>
@@ -2762,7 +2756,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B11">
         <v>4</v>
@@ -2794,7 +2788,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B12">
         <v>2</v>
@@ -2826,7 +2820,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B13">
         <v>5</v>
@@ -5175,16 +5169,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5194,21 +5187,15 @@
       <c r="C1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>138</v>
       </c>
       <c r="B2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D2">
+        <v>164</v>
+      </c>
+      <c r="C2">
         <v>5</v>
       </c>
     </row>
@@ -5234,48 +5221,48 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="J2">
         <v>80</v>
@@ -5289,7 +5276,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="J3">
         <v>90</v>
@@ -5303,7 +5290,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J4">
         <v>78</v>
@@ -5337,48 +5324,48 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B2">
         <v>2.5</v>
@@ -5404,7 +5391,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B3">
         <v>1.25</v>
@@ -5430,7 +5417,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -5476,48 +5463,48 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -5540,7 +5527,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D3">
         <v>4</v>
@@ -5560,7 +5547,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B4">
         <v>20</v>
@@ -5586,7 +5573,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D5">
         <v>8</v>
@@ -5606,7 +5593,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -5617,7 +5604,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -5646,7 +5633,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -5678,7 +5665,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B9">
         <v>5</v>
@@ -5701,7 +5688,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B10">
         <v>2</v>
@@ -5724,7 +5711,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B11">
         <v>4</v>
@@ -5750,7 +5737,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -5776,7 +5763,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B13">
         <v>5</v>

</xml_diff>

<commit_message>
some balance changes on armor
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="equipment-weapons" sheetId="1" state="visible" r:id="rId2"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="193">
   <si>
     <t xml:space="preserve">baseItem</t>
   </si>
@@ -274,19 +274,40 @@
     <t xml:space="preserve">Cloth</t>
   </si>
   <si>
-    <t xml:space="preserve">Cape</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cloak</t>
   </si>
   <si>
     <t xml:space="preserve">Robe</t>
   </si>
   <si>
-    <t xml:space="preserve">Kevlar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LeatherArmor</t>
+    <t xml:space="preserve">OfficersRobe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MageRobe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HeadGear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HeadGearCloth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bandana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PaddedCap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ribbon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WizardHat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LeatherVest</t>
   </si>
   <si>
     <t xml:space="preserve">BodyArmorLeather</t>
@@ -295,13 +316,28 @@
     <t xml:space="preserve">Leather</t>
   </si>
   <si>
-    <t xml:space="preserve">HardLeatherArmor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">StuddedLeatherArmor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DemonsaurArmor</t>
+    <t xml:space="preserve">HardLeather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StuddedLeather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DemonsaurLeather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eyepatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HeadGearLeather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LeatherHat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LeatherHelm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DemonsaurHelm</t>
   </si>
   <si>
     <t xml:space="preserve">RingMail</t>
@@ -316,15 +352,30 @@
     <t xml:space="preserve">ChainMail</t>
   </si>
   <si>
-    <t xml:space="preserve">ScaleMail</t>
-  </si>
-  <si>
     <t xml:space="preserve">SplintMail</t>
   </si>
   <si>
+    <t xml:space="preserve">FeatherMail</t>
+  </si>
+  <si>
     <t xml:space="preserve">OhmushellMail</t>
   </si>
   <si>
+    <t xml:space="preserve">Hairpin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HeadGearMail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skullcap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OhmushellMask</t>
+  </si>
+  <si>
     <t xml:space="preserve">BreastPlate</t>
   </si>
   <si>
@@ -341,60 +392,6 @@
   </si>
   <si>
     <t xml:space="preserve">FullPlate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ShardPlate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HeadGear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HeadGearCloth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bandana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PaddedCap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ribbon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WizardHat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eyepatch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HeadGearLeather</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LeatherHat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LeatherHelm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DemonsaurHelm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hairpin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HeadGearMail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skullcap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OhmushellMask</t>
   </si>
   <si>
     <t xml:space="preserve">Circlet</t>
@@ -693,7 +690,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -703,6 +700,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2251,48 +2256,48 @@
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>7</v>
@@ -2321,7 +2326,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>10</v>
@@ -2344,7 +2349,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>14</v>
@@ -2361,7 +2366,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>6</v>
@@ -2378,7 +2383,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>10</v>
@@ -2386,7 +2391,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>8</v>
@@ -2415,7 +2420,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>3</v>
@@ -2447,7 +2452,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>5</v>
@@ -2476,7 +2481,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -2505,7 +2510,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>4</v>
@@ -2537,7 +2542,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
@@ -2569,7 +2574,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>5</v>
@@ -2615,15 +2620,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
-  <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:N1048576"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="9" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="6.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="7.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="6.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="7.12"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2670,7 +2683,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>77</v>
       </c>
@@ -2686,11 +2699,11 @@
       <c r="E2" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <v>6</v>
+      <c r="F2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>80</v>
@@ -2699,7 +2712,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -2715,11 +2728,11 @@
       <c r="E3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>10</v>
+      <c r="F3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>80</v>
@@ -2727,8 +2740,11 @@
       <c r="I3" s="1" t="n">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L3" s="3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>82</v>
       </c>
@@ -2744,11 +2760,11 @@
       <c r="E4" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>14</v>
+      <c r="F4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>8</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>80</v>
@@ -2756,11 +2772,11 @@
       <c r="I4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="L4" s="1" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L4" s="3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>83</v>
       </c>
@@ -2776,11 +2792,11 @@
       <c r="E5" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="F5" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>22</v>
+      <c r="F5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>80</v>
@@ -2788,11 +2804,11 @@
       <c r="I5" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="L5" s="1" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L5" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>84</v>
       </c>
@@ -2808,11 +2824,11 @@
       <c r="E6" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>40</v>
+      <c r="F6" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>80</v>
@@ -2820,770 +2836,665 @@
       <c r="I6" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="L6" s="1" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="L6" s="3" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="G7" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="H7" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="K7" s="1" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="D8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" s="1" t="n">
+      <c r="C9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="M9" s="0"/>
+      <c r="N9" s="0"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="M10" s="0"/>
+      <c r="N10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="K8" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="1" t="n">
+      <c r="E12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E9" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I9" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="K9" s="1" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>55</v>
-      </c>
-      <c r="G10" s="1" t="n">
-        <v>65</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I10" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="G12" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I12" s="1" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="D11" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="G11" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I11" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="J11" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="K11" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D12" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="G12" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I12" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="J12" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="F13" s="1" t="n">
-        <v>34</v>
-      </c>
-      <c r="G13" s="1" t="n">
-        <v>45</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I13" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="K13" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="L13" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="F14" s="1" t="n">
-        <v>48</v>
-      </c>
-      <c r="G14" s="1" t="n">
-        <v>60</v>
+        <v>5</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="K14" s="1" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="J14" s="4"/>
+      <c r="K14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L14" s="4"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D15" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I15" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="J15" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="E15" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F15" s="1" t="n">
-        <v>65</v>
-      </c>
-      <c r="G15" s="1" t="n">
-        <v>80</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="I15" s="1" t="n">
-        <v>52</v>
-      </c>
-      <c r="J15" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K15" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="L15" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K15" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L15" s="4"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="G16" s="1" t="n">
-        <v>38</v>
+        <v>8</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="J16" s="1" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>24</v>
+      </c>
+      <c r="J16" s="4"/>
+      <c r="K16" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="L16" s="4"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="G17" s="1" t="n">
-        <v>45</v>
+        <v>10</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>19</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="J17" s="1" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D18" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="F18" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="G18" s="1" t="n">
-        <v>60</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I18" s="1" t="n">
-        <v>34</v>
-      </c>
-      <c r="J18" s="1" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0"/>
+      <c r="B18" s="0"/>
+      <c r="C18" s="0"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
+      <c r="J18" s="0"/>
+      <c r="K18" s="0"/>
+      <c r="L18" s="0"/>
+      <c r="M18" s="0"/>
+      <c r="N18" s="0"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>99</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="L19" s="0"/>
+      <c r="M19" s="0"/>
+      <c r="N19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="I19" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="J19" s="1" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="B20" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>99</v>
       </c>
       <c r="D20" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I20" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="L20" s="0"/>
+      <c r="M20" s="0"/>
+      <c r="N20" s="0"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="L21" s="0"/>
+      <c r="M21" s="0"/>
+      <c r="N21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="E22" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="F22" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="F20" s="1" t="n">
-        <v>80</v>
-      </c>
-      <c r="G20" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I20" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="J20" s="1" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="G22" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="L22" s="0"/>
+      <c r="M22" s="0"/>
+      <c r="N22" s="0"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0"/>
+      <c r="B23" s="0"/>
+      <c r="C23" s="0"/>
+      <c r="D23" s="0"/>
+      <c r="E23" s="0"/>
+      <c r="F23" s="0"/>
+      <c r="G23" s="0"/>
+      <c r="H23" s="0"/>
+      <c r="I23" s="0"/>
+      <c r="J23" s="0"/>
+      <c r="K23" s="0"/>
+      <c r="L23" s="0"/>
+      <c r="M23" s="0"/>
+      <c r="N23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="I24" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K24" s="4"/>
+      <c r="L24" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="M24" s="0"/>
+      <c r="N24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="B25" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I25" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="L25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="1" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
+      <c r="B26" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="K26" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="L26" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D22" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="F22" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I22" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="L22" s="1" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="B27" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I27" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E23" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="F23" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="G23" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I23" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="L23" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="B28" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="I28" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="L28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0"/>
+      <c r="B29" s="0"/>
+      <c r="C29" s="0"/>
+      <c r="D29" s="0"/>
+      <c r="E29" s="0"/>
+      <c r="F29" s="0"/>
+      <c r="G29" s="0"/>
+      <c r="H29" s="0"/>
+      <c r="I29" s="0"/>
+      <c r="J29" s="0"/>
+      <c r="K29" s="0"/>
+      <c r="L29" s="0"/>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D24" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I24" s="1" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="E25" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F25" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="G25" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="H25" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I25" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="L25" s="1" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D26" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I26" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="K26" s="1" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E27" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="F27" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="G27" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I27" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="K27" s="1" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E28" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="F28" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="G28" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I28" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="K28" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="E29" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F29" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="G29" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="I29" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="K29" s="1" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>3</v>
@@ -3598,21 +3509,21 @@
         <v>2</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="I30" s="1" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D31" s="1" t="n">
         <v>4</v>
@@ -3624,30 +3535,24 @@
         <v>8</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="I31" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="J31" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="K31" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D32" s="1" t="n">
         <v>5</v>
@@ -3656,36 +3561,27 @@
         <v>8</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="I32" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="J32" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="K32" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="L32" s="1" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>7</v>
@@ -3694,152 +3590,505 @@
         <v>10</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="I33" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="J33" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="K33" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="L33" s="1" t="n">
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0"/>
+      <c r="B34" s="0"/>
+      <c r="C34" s="0"/>
+      <c r="D34" s="0"/>
+      <c r="E34" s="0"/>
+      <c r="F34" s="0"/>
+      <c r="G34" s="0"/>
+      <c r="H34" s="0"/>
+      <c r="I34" s="0"/>
+      <c r="J34" s="0"/>
+      <c r="K34" s="0"/>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I35" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="J35" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="K35" s="4"/>
+      <c r="L35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I36" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I37" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="K37" s="4"/>
+      <c r="L37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="E38" s="1" t="n">
         <v>9</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="s">
+      <c r="F38" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I38" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="K38" s="4"/>
+      <c r="L38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0"/>
+      <c r="B39" s="0"/>
+      <c r="C39" s="0"/>
+      <c r="D39" s="0"/>
+      <c r="E39" s="0"/>
+      <c r="F39" s="0"/>
+      <c r="G39" s="0"/>
+      <c r="H39" s="0"/>
+      <c r="I39" s="0"/>
+      <c r="J39" s="0"/>
+      <c r="K39" s="0"/>
+      <c r="L39" s="0"/>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C34" s="1" t="s">
+      <c r="D40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="G40" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I40" s="1" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D34" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="1" t="n">
+      <c r="B41" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D41" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F34" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="G34" s="1" t="n">
+      <c r="E41" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="F41" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="H34" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I34" s="1" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
+      <c r="G41" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I41" s="1" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D35" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E35" s="1" t="n">
+      <c r="B42" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D42" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="F35" s="1" t="n">
+      <c r="E42" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I42" s="1" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="G35" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I35" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="J35" s="1" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D36" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E36" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="F36" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="G36" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I36" s="1" t="n">
-        <v>31</v>
-      </c>
-      <c r="J36" s="1" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D37" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="E37" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="F37" s="1" t="n">
+      <c r="F43" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="G37" s="1" t="n">
+      <c r="G43" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="H37" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="I37" s="1" t="n">
+      <c r="H43" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="I43" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="J37" s="1" t="n">
-        <v>19</v>
-      </c>
-    </row>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0"/>
+      <c r="B44" s="0"/>
+      <c r="C44" s="0"/>
+      <c r="D44" s="0"/>
+      <c r="E44" s="0"/>
+      <c r="F44" s="0"/>
+      <c r="G44" s="0"/>
+      <c r="H44" s="0"/>
+      <c r="I44" s="0"/>
+      <c r="J44" s="0"/>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0"/>
+      <c r="B46" s="0"/>
+      <c r="C46" s="0"/>
+      <c r="D46" s="0"/>
+      <c r="E46" s="0"/>
+      <c r="F46" s="0"/>
+      <c r="G46" s="0"/>
+      <c r="H46" s="0"/>
+      <c r="I46" s="0"/>
+      <c r="J46" s="0"/>
+      <c r="K46" s="0"/>
+      <c r="L46" s="0"/>
+      <c r="M46" s="0"/>
+      <c r="N46" s="0"/>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0"/>
+      <c r="B47" s="0"/>
+      <c r="C47" s="0"/>
+      <c r="D47" s="0"/>
+      <c r="E47" s="0"/>
+      <c r="F47" s="0"/>
+      <c r="G47" s="0"/>
+      <c r="H47" s="0"/>
+      <c r="I47" s="0"/>
+      <c r="J47" s="0"/>
+      <c r="K47" s="0"/>
+      <c r="L47" s="0"/>
+      <c r="M47" s="0"/>
+      <c r="N47" s="0"/>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0"/>
+      <c r="B48" s="0"/>
+      <c r="C48" s="0"/>
+      <c r="D48" s="0"/>
+      <c r="E48" s="0"/>
+      <c r="F48" s="0"/>
+      <c r="G48" s="0"/>
+      <c r="H48" s="0"/>
+      <c r="I48" s="0"/>
+      <c r="J48" s="0"/>
+      <c r="K48" s="0"/>
+      <c r="L48" s="0"/>
+      <c r="M48" s="0"/>
+      <c r="N48" s="0"/>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0"/>
+      <c r="B49" s="0"/>
+      <c r="C49" s="0"/>
+      <c r="D49" s="0"/>
+      <c r="E49" s="0"/>
+      <c r="F49" s="0"/>
+      <c r="G49" s="0"/>
+      <c r="H49" s="0"/>
+      <c r="I49" s="0"/>
+      <c r="J49" s="0"/>
+      <c r="K49" s="0"/>
+      <c r="L49" s="0"/>
+      <c r="M49" s="0"/>
+      <c r="N49" s="0"/>
+    </row>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0"/>
+      <c r="B52" s="0"/>
+      <c r="C52" s="0"/>
+      <c r="D52" s="0"/>
+      <c r="E52" s="0"/>
+      <c r="F52" s="0"/>
+      <c r="G52" s="0"/>
+      <c r="H52" s="0"/>
+      <c r="I52" s="0"/>
+      <c r="J52" s="0"/>
+      <c r="K52" s="0"/>
+      <c r="L52" s="0"/>
+    </row>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0"/>
+      <c r="B53" s="0"/>
+      <c r="C53" s="0"/>
+      <c r="D53" s="0"/>
+      <c r="E53" s="0"/>
+      <c r="F53" s="0"/>
+      <c r="G53" s="0"/>
+      <c r="H53" s="0"/>
+      <c r="I53" s="0"/>
+      <c r="J53" s="0"/>
+      <c r="K53" s="0"/>
+      <c r="L53" s="0"/>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0"/>
+      <c r="B54" s="0"/>
+      <c r="C54" s="0"/>
+      <c r="D54" s="0"/>
+      <c r="E54" s="0"/>
+      <c r="F54" s="0"/>
+      <c r="G54" s="0"/>
+      <c r="H54" s="0"/>
+      <c r="I54" s="0"/>
+      <c r="J54" s="0"/>
+      <c r="K54" s="0"/>
+      <c r="L54" s="0"/>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0"/>
+      <c r="B55" s="0"/>
+      <c r="C55" s="0"/>
+      <c r="D55" s="0"/>
+      <c r="E55" s="0"/>
+      <c r="F55" s="0"/>
+      <c r="G55" s="0"/>
+      <c r="H55" s="0"/>
+      <c r="I55" s="0"/>
+      <c r="J55" s="0"/>
+      <c r="K55" s="0"/>
+      <c r="L55" s="0"/>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0"/>
+      <c r="B56" s="0"/>
+      <c r="C56" s="0"/>
+      <c r="D56" s="0"/>
+      <c r="E56" s="0"/>
+      <c r="F56" s="0"/>
+      <c r="G56" s="0"/>
+      <c r="H56" s="0"/>
+      <c r="I56" s="0"/>
+      <c r="J56" s="0"/>
+      <c r="K56" s="0"/>
+      <c r="L56" s="0"/>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0"/>
+      <c r="B58" s="0"/>
+      <c r="C58" s="0"/>
+      <c r="D58" s="0"/>
+      <c r="E58" s="0"/>
+      <c r="F58" s="0"/>
+      <c r="G58" s="0"/>
+      <c r="H58" s="0"/>
+      <c r="I58" s="0"/>
+      <c r="J58" s="0"/>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0"/>
+      <c r="B59" s="0"/>
+      <c r="C59" s="0"/>
+      <c r="D59" s="0"/>
+      <c r="E59" s="0"/>
+      <c r="F59" s="0"/>
+      <c r="G59" s="0"/>
+      <c r="H59" s="0"/>
+      <c r="I59" s="0"/>
+      <c r="J59" s="0"/>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="0"/>
+      <c r="B60" s="0"/>
+      <c r="C60" s="0"/>
+      <c r="D60" s="0"/>
+      <c r="E60" s="0"/>
+      <c r="F60" s="0"/>
+      <c r="G60" s="0"/>
+      <c r="H60" s="0"/>
+      <c r="I60" s="0"/>
+      <c r="J60" s="0"/>
+    </row>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="0"/>
+      <c r="B61" s="0"/>
+      <c r="C61" s="0"/>
+      <c r="D61" s="0"/>
+      <c r="E61" s="0"/>
+      <c r="F61" s="0"/>
+      <c r="G61" s="0"/>
+      <c r="H61" s="0"/>
+      <c r="I61" s="0"/>
+      <c r="J61" s="0"/>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="0"/>
+      <c r="B62" s="0"/>
+      <c r="C62" s="0"/>
+      <c r="D62" s="0"/>
+      <c r="E62" s="0"/>
+      <c r="F62" s="0"/>
+      <c r="G62" s="0"/>
+      <c r="H62" s="0"/>
+      <c r="I62" s="0"/>
+      <c r="J62" s="0"/>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3886,7 +4135,7 @@
         <v>75</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>9</v>
@@ -3909,10 +4158,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>0</v>
@@ -3927,7 +4176,7 @@
         <v>2</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>8</v>
@@ -3935,10 +4184,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>1</v>
@@ -3953,7 +4202,7 @@
         <v>6</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H3" s="1" t="n">
         <v>16</v>
@@ -3961,10 +4210,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>2</v>
@@ -3979,7 +4228,7 @@
         <v>18</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H4" s="1" t="n">
         <v>22</v>
@@ -3990,10 +4239,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>3</v>
@@ -4008,7 +4257,7 @@
         <v>32</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>18</v>
@@ -4022,10 +4271,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C6" s="1" t="n">
         <v>4</v>
@@ -4040,7 +4289,7 @@
         <v>41</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H6" s="1" t="n">
         <v>20</v>
@@ -4054,10 +4303,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C7" s="1" t="n">
         <v>5</v>
@@ -4072,7 +4321,7 @@
         <v>48</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H7" s="1" t="n">
         <v>18</v>
@@ -4086,10 +4335,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>5</v>
@@ -4104,7 +4353,7 @@
         <v>55</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H8" s="1" t="n">
         <v>15</v>
@@ -4118,10 +4367,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>6</v>
@@ -4136,7 +4385,7 @@
         <v>75</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>24</v>
@@ -4150,10 +4399,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>7</v>
@@ -4168,7 +4417,7 @@
         <v>80</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H10" s="1" t="n">
         <v>25</v>
@@ -4179,10 +4428,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>8</v>
@@ -4197,7 +4446,7 @@
         <v>100</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>28</v>
@@ -4211,10 +4460,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>8</v>
@@ -4229,7 +4478,7 @@
         <v>110</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H12" s="1" t="n">
         <v>28</v>
@@ -4303,13 +4552,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>3</v>
@@ -4320,13 +4569,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>3</v>
@@ -4377,52 +4626,52 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4602,7 +4851,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>3</v>
@@ -4640,7 +4889,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>5</v>
@@ -4678,7 +4927,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>3</v>
@@ -4710,7 +4959,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>5</v>
@@ -4748,7 +4997,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>3</v>
@@ -4789,7 +5038,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>5</v>
@@ -4830,7 +5079,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
@@ -4865,7 +5114,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>5</v>
@@ -4903,7 +5152,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
@@ -4971,18 +5220,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>5</v>
@@ -5018,48 +5267,48 @@
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J2" s="1" t="n">
         <v>80</v>
@@ -5073,7 +5322,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J3" s="1" t="n">
         <v>90</v>
@@ -5087,7 +5336,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J4" s="1" t="n">
         <v>78</v>
@@ -5129,48 +5378,48 @@
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>2.5</v>
@@ -5196,7 +5445,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>1.25</v>
@@ -5222,7 +5471,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
@@ -5276,48 +5525,48 @@
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>100</v>
@@ -5340,7 +5589,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>4</v>
@@ -5360,7 +5609,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>20</v>
@@ -5386,7 +5635,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>8</v>
@@ -5406,7 +5655,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>10</v>
@@ -5417,7 +5666,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>2</v>
@@ -5446,7 +5695,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>2</v>
@@ -5478,7 +5727,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>50</v>
@@ -5501,7 +5750,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>2</v>
@@ -5524,7 +5773,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>4</v>
@@ -5550,7 +5799,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>1</v>
@@ -5576,7 +5825,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
moving accuracy caluclations into own folders
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="attack-damage" sheetId="1" state="visible" r:id="rId2"/>
@@ -16071,7 +16071,7 @@
         <v>22</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16106,7 +16106,7 @@
         <v>18</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16141,7 +16141,7 @@
         <v>20</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16208,7 +16208,7 @@
         <v>15</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16243,10 +16243,10 @@
         <v>17</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16281,10 +16281,10 @@
         <v>24</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16319,10 +16319,10 @@
         <v>25</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16389,7 +16389,7 @@
         <v>13</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16424,10 +16424,10 @@
         <v>25</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16462,13 +16462,13 @@
         <v>20</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16503,10 +16503,10 @@
         <v>12</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16541,10 +16541,10 @@
         <v>9</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16579,7 +16579,7 @@
         <v>10</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16614,7 +16614,7 @@
         <v>14</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16649,7 +16649,7 @@
         <v>18</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16684,7 +16684,7 @@
         <v>24</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16783,10 +16783,10 @@
         <v>11</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16821,7 +16821,7 @@
         <v>15</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16856,10 +16856,10 @@
         <v>16</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="L26" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16894,7 +16894,7 @@
         <v>18</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16929,10 +16929,10 @@
         <v>21</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16967,10 +16967,10 @@
         <v>19</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L29" s="7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17005,10 +17005,10 @@
         <v>18</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M30" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17043,10 +17043,10 @@
         <v>23</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M31" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17081,10 +17081,10 @@
         <v>28</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="L32" s="7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17119,7 +17119,7 @@
         <v>40</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17154,7 +17154,7 @@
         <v>16</v>
       </c>
       <c r="M34" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17189,7 +17189,7 @@
         <v>19</v>
       </c>
       <c r="M35" s="7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17224,7 +17224,7 @@
         <v>24</v>
       </c>
       <c r="M36" s="7" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17259,7 +17259,7 @@
         <v>15</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17294,10 +17294,10 @@
         <v>16</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17332,10 +17332,10 @@
         <v>26</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L39" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17370,10 +17370,10 @@
         <v>25</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="L40" s="7" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17408,10 +17408,10 @@
         <v>11</v>
       </c>
       <c r="L41" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="M41" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
seeded rng for dummy sampling to avoid noise leading to allocating non-contributing attribute
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -848,47 +848,47 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -15919,12 +15919,15 @@
   <dimension ref="A1:O41"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="23.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="35.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="7" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="7" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="13.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="16.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="20.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="7.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="7.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="8.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="9.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="25.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="7" width="26.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="7" width="10"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
thinking of how to auto generate equipment attribute requirements
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="attack-damage" sheetId="1" state="visible" r:id="rId2"/>
@@ -843,7 +843,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -889,6 +889,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -15127,8 +15131,8 @@
       <c r="I14" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="K14" s="11" t="n">
-        <v>10</v>
+      <c r="K14" s="12" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15926,7 +15930,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="7.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="8.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="9.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="25.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="25.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="7" width="26.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="7" width="10"/>
   </cols>

</xml_diff>

<commit_message>
about to write new thing
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -843,7 +843,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -894,6 +894,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -15163,11 +15167,11 @@
       <c r="I15" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="J15" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K15" s="11" t="n">
-        <v>8</v>
+      <c r="J15" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15198,8 +15202,8 @@
       <c r="I16" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="K16" s="11" t="n">
-        <v>33</v>
+      <c r="K16" s="12" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15230,12 +15234,10 @@
       <c r="I17" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="K17" s="11" t="n">
-        <v>21</v>
-      </c>
-      <c r="L17" s="11" t="n">
-        <v>21</v>
-      </c>
+      <c r="K17" s="13" t="n">
+        <v>55</v>
+      </c>
+      <c r="L17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15520,8 +15522,11 @@
       <c r="I28" s="7" t="n">
         <v>52</v>
       </c>
-      <c r="K28" s="11" t="n">
-        <v>55</v>
+      <c r="K28" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="L28" s="12" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
combine balance packages, generate equipment requirements from studies
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -12,15 +12,16 @@
     <sheet name="by-level-attribute-visual" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="balancing" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="equipment-armor" sheetId="4" state="visible" r:id="rId5"/>
-    <sheet name="equipment-weapons" sheetId="5" state="visible" r:id="rId6"/>
-    <sheet name="equipment-shields" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="equipment-jewelry" sheetId="7" state="visible" r:id="rId8"/>
-    <sheet name="equipment-affix-profiles" sheetId="8" state="visible" r:id="rId9"/>
-    <sheet name="equipment-affix-overrides" sheetId="9" state="visible" r:id="rId10"/>
-    <sheet name="class-starting-attributes" sheetId="10" state="visible" r:id="rId11"/>
-    <sheet name="class-attributes-per-level" sheetId="11" state="visible" r:id="rId12"/>
-    <sheet name="monster-starting-attributes" sheetId="12" state="visible" r:id="rId13"/>
-    <sheet name="monster-attributes-per-level" sheetId="13" state="visible" r:id="rId14"/>
+    <sheet name="equipment-requirement-targets" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="equipment-weapons" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="equipment-shields" sheetId="7" state="visible" r:id="rId8"/>
+    <sheet name="equipment-jewelry" sheetId="8" state="visible" r:id="rId9"/>
+    <sheet name="equipment-affix-profiles" sheetId="9" state="visible" r:id="rId10"/>
+    <sheet name="equipment-affix-overrides" sheetId="10" state="visible" r:id="rId11"/>
+    <sheet name="class-starting-attributes" sheetId="11" state="visible" r:id="rId12"/>
+    <sheet name="class-attributes-per-level" sheetId="12" state="visible" r:id="rId13"/>
+    <sheet name="monster-starting-attributes" sheetId="13" state="visible" r:id="rId14"/>
+    <sheet name="monster-attributes-per-level" sheetId="14" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="ArmorClassModifier" vbProcedure="false">balancing!$B$9</definedName>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="239">
   <si>
     <t xml:space="preserve">minDmg</t>
   </si>
@@ -231,6 +232,9 @@
     <t xml:space="preserve">Cloak</t>
   </si>
   <si>
+    <t xml:space="preserve">equipmentType | baseItem | study | attributes | weaponSpecialty | mainClass | supportClass | availabilityPercentile |</t>
+  </si>
+  <si>
     <t xml:space="preserve">Robe</t>
   </si>
   <si>
@@ -354,6 +358,39 @@
     <t xml:space="preserve">GreatHelm</t>
   </si>
   <si>
+    <t xml:space="preserve">study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">attributes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">weaponSpecialty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mainClass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supportClass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">availabilityPercentile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackDamageMixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dexterity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TwoHandedRanged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rogue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warrior</t>
+  </si>
+  <si>
     <t xml:space="preserve">damageClassificationsCount</t>
   </si>
   <si>
@@ -519,9 +556,6 @@
     <t xml:space="preserve">TwoHandedRangedWeapon</t>
   </si>
   <si>
-    <t xml:space="preserve">TwoHandedRanged</t>
-  </si>
-  <si>
     <t xml:space="preserve">RecurveBow</t>
   </si>
   <si>
@@ -657,9 +691,6 @@
     <t xml:space="preserve">Strength</t>
   </si>
   <si>
-    <t xml:space="preserve">Dexterity</t>
-  </si>
-  <si>
     <t xml:space="preserve">Spirit</t>
   </si>
   <si>
@@ -688,12 +719,6 @@
   </si>
   <si>
     <t xml:space="preserve">Mp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Warrior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rogue</t>
   </si>
   <si>
     <t xml:space="preserve">Mage</t>
@@ -746,7 +771,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -781,6 +806,12 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -843,7 +874,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -856,7 +887,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -864,7 +895,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -896,7 +927,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -12504,108 +12559,34 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="7" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="7" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="7" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="10"/>
   </cols>
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>202</v>
+        <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="J1" s="10" t="s">
         <v>211</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>213</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="L2" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="M2" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>90</v>
-      </c>
-      <c r="L3" s="7" t="n">
-        <v>18</v>
-      </c>
-      <c r="M3" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>78</v>
-      </c>
-      <c r="L4" s="7" t="n">
-        <v>15</v>
-      </c>
-      <c r="M4" s="7" t="n">
-        <v>4</v>
+        <v>186</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -12638,121 +12619,94 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>204</v>
+        <v>111</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>215</v>
-      </c>
-      <c r="B2" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="C2" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D2" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E2" s="7" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="F2" s="7" t="n">
-        <v>0.75</v>
+        <v>114</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>80</v>
       </c>
       <c r="L2" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="M2" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="M2" s="7" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E3" s="7" t="n">
+        <v>113</v>
+      </c>
+      <c r="G3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F3" s="7" t="n">
-        <v>1.5</v>
+      <c r="J3" s="7" t="n">
+        <v>90</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.5</v>
+        <v>18</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="B4" s="7" t="n">
+        <v>225</v>
+      </c>
+      <c r="G4" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="7" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="D4" s="7" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>0.75</v>
+      <c r="J4" s="7" t="n">
+        <v>78</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -12771,10 +12725,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="7" width="10"/>
@@ -12785,337 +12739,121 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>208</v>
-      </c>
       <c r="H1" s="10" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>219</v>
+        <v>114</v>
       </c>
       <c r="B2" s="7" t="n">
-        <v>100</v>
+        <v>2.5</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="E2" s="7" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="7" t="n">
         <v>1</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H2" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="L2" s="7" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>220</v>
+        <v>113</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>2.5</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>4</v>
+        <v>0.75</v>
       </c>
       <c r="E3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="G3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>60</v>
-      </c>
       <c r="L3" s="7" t="n">
-        <v>3</v>
+        <v>1.5</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>1.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B4" s="7" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>20</v>
+        <v>1.75</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>0</v>
+        <v>2.5</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0.75</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>223</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="B7" s="7" t="n">
+      <c r="M4" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="L7" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="M7" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>80</v>
-      </c>
-      <c r="L8" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="M8" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="B9" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="B10" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="L10" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="B11" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="L11" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>65</v>
-      </c>
-      <c r="L12" s="7" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="B13" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="L13" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="M13" s="7" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -13148,48 +12886,411 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>208</v>
-      </c>
       <c r="H1" s="10" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="7" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="7" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="7" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="7" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" s="10" t="s">
         <v>219</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>227</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>7</v>
@@ -13218,7 +13319,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>10</v>
@@ -13241,7 +13342,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>14</v>
@@ -13258,7 +13359,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>6</v>
@@ -13275,7 +13376,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>10</v>
@@ -13283,7 +13384,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>8</v>
@@ -13312,7 +13413,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>3</v>
@@ -13344,7 +13445,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>5</v>
@@ -13373,7 +13474,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>4</v>
@@ -13402,7 +13503,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>4</v>
@@ -13434,7 +13535,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -13466,7 +13567,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>5</v>
@@ -14739,7 +14840,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N1048576"/>
+  <dimension ref="A1:O1048576"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="16.43"/>
@@ -14863,10 +14964,13 @@
       <c r="L3" s="11" t="n">
         <v>15</v>
       </c>
+      <c r="O3" s="7" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>59</v>
@@ -14898,7 +15002,7 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>59</v>
@@ -14930,7 +15034,7 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>59</v>
@@ -14963,13 +15067,13 @@
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>1</v>
@@ -14992,13 +15096,13 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>68</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>2</v>
@@ -15021,13 +15125,13 @@
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>3</v>
@@ -15050,13 +15154,13 @@
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>5</v>
@@ -15079,13 +15183,13 @@
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>7</v>
@@ -15109,13 +15213,13 @@
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>3</v>
@@ -15135,19 +15239,17 @@
       <c r="I14" s="7" t="n">
         <v>16</v>
       </c>
-      <c r="K14" s="12" t="n">
-        <v>16</v>
-      </c>
+      <c r="K14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>5</v>
@@ -15176,13 +15278,13 @@
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>6</v>
@@ -15208,13 +15310,13 @@
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>8</v>
@@ -15237,18 +15339,18 @@
       <c r="K17" s="13" t="n">
         <v>55</v>
       </c>
-      <c r="L17" s="0"/>
+      <c r="L17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>1</v>
@@ -15271,13 +15373,13 @@
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>79</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>3</v>
@@ -15300,13 +15402,13 @@
     </row>
     <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>4</v>
@@ -15329,13 +15431,13 @@
     </row>
     <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>9</v>
@@ -15359,13 +15461,13 @@
     <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>3</v>
@@ -15394,13 +15496,13 @@
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>4</v>
@@ -15429,13 +15531,13 @@
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D26" s="7" t="n">
         <v>5</v>
@@ -15461,13 +15563,13 @@
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>5</v>
@@ -15496,13 +15598,13 @@
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>8</v>
@@ -15532,13 +15634,13 @@
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>3</v>
@@ -15561,13 +15663,13 @@
     </row>
     <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>89</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>4</v>
@@ -15590,13 +15692,13 @@
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>5</v>
@@ -15619,13 +15721,13 @@
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>7</v>
@@ -15649,13 +15751,13 @@
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>2</v>
@@ -15681,13 +15783,13 @@
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D36" s="7" t="n">
         <v>4</v>
@@ -15713,13 +15815,13 @@
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D37" s="7" t="n">
         <v>5</v>
@@ -15745,13 +15847,13 @@
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>59</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D38" s="7" t="n">
         <v>8</v>
@@ -15778,13 +15880,13 @@
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>2</v>
@@ -15807,13 +15909,13 @@
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C41" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>99</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>4</v>
@@ -15836,13 +15938,13 @@
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D42" s="7" t="n">
         <v>6</v>
@@ -15865,13 +15967,13 @@
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>9</v>
@@ -15925,6 +16027,456 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:O1048576"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="14.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="15" width="17.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="15" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="15" width="9.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="15" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="15" width="14.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="15" width="9.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="15" width="6.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="15" width="7.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="15" width="7.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="15" width="6.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="15" width="7.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="15" min="15" style="7" width="11.55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="10"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="O3" s="0"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="L4" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="L5" s="18"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="L6" s="18"/>
+    </row>
+    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H14" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K14" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
+    </row>
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="K16" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="J24" s="18"/>
+      <c r="L24" s="18"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="K26" s="18"/>
+    </row>
+    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="18"/>
+    </row>
+    <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="K28" s="18"/>
+      <c r="L28" s="18"/>
+    </row>
+    <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="J35" s="18"/>
+    </row>
+    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="J36" s="18"/>
+    </row>
+    <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="J37" s="18"/>
+    </row>
+    <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="J38" s="18"/>
+    </row>
+    <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="53" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="55" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="57" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="60" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:O41"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -15963,10 +16515,10 @@
         <v>1</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="J1" s="10" t="s">
         <v>52</v>
@@ -15989,13 +16541,13 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>0</v>
@@ -16013,7 +16565,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>8</v>
@@ -16021,13 +16573,13 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>1</v>
@@ -16045,7 +16597,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>14</v>
@@ -16053,13 +16605,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>2</v>
@@ -16077,7 +16629,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>22</v>
@@ -16088,13 +16640,13 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>4</v>
@@ -16112,7 +16664,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>18</v>
@@ -16123,13 +16675,13 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>8</v>
@@ -16147,7 +16699,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>20</v>
@@ -16158,13 +16710,13 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>0</v>
@@ -16182,7 +16734,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>7</v>
@@ -16190,13 +16742,13 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>2</v>
@@ -16214,7 +16766,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>15</v>
@@ -16225,13 +16777,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>3</v>
@@ -16249,7 +16801,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>17</v>
@@ -16263,13 +16815,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>6</v>
@@ -16287,7 +16839,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>24</v>
@@ -16301,13 +16853,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>8</v>
@@ -16325,7 +16877,7 @@
         <v>2</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>25</v>
@@ -16339,13 +16891,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>1</v>
@@ -16363,7 +16915,7 @@
         <v>2</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>9</v>
@@ -16371,13 +16923,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>3</v>
@@ -16395,7 +16947,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>13</v>
@@ -16406,13 +16958,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>6</v>
@@ -16430,7 +16982,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>25</v>
@@ -16444,13 +16996,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>5</v>
@@ -16468,7 +17020,7 @@
         <v>2</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>20</v>
@@ -16485,13 +17037,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>5</v>
@@ -16509,7 +17061,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>12</v>
@@ -16523,13 +17075,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>2</v>
@@ -16547,7 +17099,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>9</v>
@@ -16561,13 +17113,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>2</v>
@@ -16585,7 +17137,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>10</v>
@@ -16596,13 +17148,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>3</v>
@@ -16620,7 +17172,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>14</v>
@@ -16631,13 +17183,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>5</v>
@@ -16655,7 +17207,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>18</v>
@@ -16666,13 +17218,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>8</v>
@@ -16690,7 +17242,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>24</v>
@@ -16701,13 +17253,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>0</v>
@@ -16725,7 +17277,7 @@
         <v>1</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>6</v>
@@ -16733,13 +17285,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>1</v>
@@ -16757,7 +17309,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>8</v>
@@ -16765,13 +17317,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>2</v>
@@ -16789,7 +17341,7 @@
         <v>1</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>11</v>
@@ -16803,13 +17355,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>2</v>
@@ -16827,7 +17379,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>15</v>
@@ -16838,13 +17390,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D26" s="7" t="n">
         <v>3</v>
@@ -16862,7 +17414,7 @@
         <v>2</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>16</v>
@@ -16876,13 +17428,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>5</v>
@@ -16900,7 +17452,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>18</v>
@@ -16911,13 +17463,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>5</v>
@@ -16935,7 +17487,7 @@
         <v>1</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>21</v>
@@ -16949,13 +17501,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>6</v>
@@ -16973,7 +17525,7 @@
         <v>2</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>19</v>
@@ -16987,13 +17539,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>7</v>
@@ -17011,7 +17563,7 @@
         <v>2</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>18</v>
@@ -17025,13 +17577,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>136</v>
-      </c>
       <c r="C31" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>8</v>
@@ -17049,7 +17601,7 @@
         <v>2</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>23</v>
@@ -17063,13 +17615,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>9</v>
@@ -17087,7 +17639,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>28</v>
@@ -17101,13 +17653,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>9</v>
@@ -17125,7 +17677,7 @@
         <v>1</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>40</v>
@@ -17136,13 +17688,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>3</v>
@@ -17160,7 +17712,7 @@
         <v>1</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>16</v>
@@ -17171,13 +17723,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>5</v>
@@ -17195,7 +17747,7 @@
         <v>1</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>19</v>
@@ -17206,13 +17758,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D36" s="7" t="n">
         <v>8</v>
@@ -17230,7 +17782,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>24</v>
@@ -17241,13 +17793,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D37" s="7" t="n">
         <v>1</v>
@@ -17265,7 +17817,7 @@
         <v>1</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>15</v>
@@ -17276,13 +17828,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D38" s="7" t="n">
         <v>3</v>
@@ -17300,7 +17852,7 @@
         <v>1</v>
       </c>
       <c r="I38" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>16</v>
@@ -17314,13 +17866,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>5</v>
@@ -17338,7 +17890,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>26</v>
@@ -17352,13 +17904,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>8</v>
@@ -17376,7 +17928,7 @@
         <v>1</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>25</v>
@@ -17390,13 +17942,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>7</v>
@@ -17414,7 +17966,7 @@
         <v>1</v>
       </c>
       <c r="I41" s="7" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>11</v>
@@ -17437,7 +17989,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -17480,7 +18032,7 @@
         <v>50</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>52</v>
@@ -17503,10 +18055,10 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>0</v>
@@ -17521,7 +18073,7 @@
         <v>2</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>8</v>
@@ -17529,10 +18081,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>1</v>
@@ -17547,7 +18099,7 @@
         <v>5</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>16</v>
@@ -17555,10 +18107,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>2</v>
@@ -17573,7 +18125,7 @@
         <v>14</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>22</v>
@@ -17581,10 +18133,10 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>3</v>
@@ -17599,7 +18151,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>18</v>
@@ -17607,10 +18159,10 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>4</v>
@@ -17625,7 +18177,7 @@
         <v>19</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>20</v>
@@ -17633,10 +18185,10 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>5</v>
@@ -17651,7 +18203,7 @@
         <v>18</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>18</v>
@@ -17659,10 +18211,10 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>5</v>
@@ -17677,7 +18229,7 @@
         <v>15</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>15</v>
@@ -17685,10 +18237,10 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>6</v>
@@ -17703,7 +18255,7 @@
         <v>23</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>24</v>
@@ -17711,10 +18263,10 @@
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>177</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>166</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>7</v>
@@ -17729,7 +18281,7 @@
         <v>28</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>25</v>
@@ -17737,10 +18289,10 @@
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>8</v>
@@ -17755,7 +18307,7 @@
         <v>24</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>28</v>
@@ -17763,10 +18315,10 @@
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>8</v>
@@ -17781,7 +18333,7 @@
         <v>28</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>28</v>
@@ -17798,7 +18350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -17849,13 +18401,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>3</v>
@@ -17866,13 +18418,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>3</v>
@@ -17892,7 +18444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -17923,57 +18475,57 @@
         <v>46</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="N1" s="10" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="O1" s="10" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="P1" s="10" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>5</v>
@@ -18008,7 +18560,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>5</v>
@@ -18046,7 +18598,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>5</v>
@@ -18069,7 +18621,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>158</v>
+        <v>112</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>5</v>
@@ -18148,7 +18700,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>3</v>
@@ -18186,7 +18738,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>5</v>
@@ -18224,7 +18776,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>3</v>
@@ -18256,7 +18808,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>5</v>
@@ -18294,7 +18846,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>3</v>
@@ -18335,7 +18887,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>5</v>
@@ -18376,7 +18928,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>3</v>
@@ -18411,7 +18963,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>5</v>
@@ -18449,7 +19001,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>5</v>
@@ -18485,52 +19037,6 @@
         <v>5</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="C2" s="7" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
generating equipment requirements from studies automatically, need more studies
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="attack-damage" sheetId="1" state="visible" r:id="rId2"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="240">
   <si>
     <t xml:space="preserve">minDmg</t>
   </si>
@@ -391,6 +391,18 @@
     <t xml:space="preserve">Warrior</t>
   </si>
   <si>
+    <t xml:space="preserve">Dexterity, Strength</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strength</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TwoHandedMelee</t>
+  </si>
+  <si>
     <t xml:space="preserve">damageClassificationsCount</t>
   </si>
   <si>
@@ -493,9 +505,6 @@
     <t xml:space="preserve">TwoHandedMeleeWeapon</t>
   </si>
   <si>
-    <t xml:space="preserve">TwoHandedMelee</t>
-  </si>
-  <si>
     <t xml:space="preserve">BoStaff</t>
   </si>
   <si>
@@ -688,9 +697,6 @@
     <t xml:space="preserve">combatantClass</t>
   </si>
   <si>
-    <t xml:space="preserve">Strength</t>
-  </si>
-  <si>
     <t xml:space="preserve">Spirit</t>
   </si>
   <si>
@@ -719,9 +725,6 @@
   </si>
   <si>
     <t xml:space="preserve">Mp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mage</t>
   </si>
   <si>
     <t xml:space="preserve">monsterType</t>
@@ -12572,18 +12575,18 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>5</v>
@@ -12619,43 +12622,43 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>214</v>
+        <v>117</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>111</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12694,7 +12697,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>225</v>
+        <v>116</v>
       </c>
       <c r="G4" s="7" t="n">
         <v>1</v>
@@ -12739,43 +12742,43 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>214</v>
+        <v>117</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>111</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12832,7 +12835,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>225</v>
+        <v>116</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>1</v>
@@ -12886,48 +12889,48 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>214</v>
+        <v>117</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>111</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>100</v>
@@ -12950,7 +12953,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>4</v>
@@ -12970,7 +12973,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>20</v>
@@ -12996,7 +12999,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>8</v>
@@ -13016,7 +13019,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>10</v>
@@ -13027,7 +13030,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>2</v>
@@ -13056,7 +13059,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>2</v>
@@ -13088,7 +13091,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>50</v>
@@ -13111,7 +13114,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>2</v>
@@ -13134,7 +13137,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>4</v>
@@ -13160,7 +13163,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>1</v>
@@ -13186,7 +13189,7 @@
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>5</v>
@@ -13249,48 +13252,48 @@
   <sheetData>
     <row r="1" s="10" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>214</v>
+        <v>117</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>111</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B2" s="7" t="n">
         <v>7</v>
@@ -13319,7 +13322,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>10</v>
@@ -13342,7 +13345,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>14</v>
@@ -13359,7 +13362,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>6</v>
@@ -13376,7 +13379,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>10</v>
@@ -13384,7 +13387,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>8</v>
@@ -13413,7 +13416,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>3</v>
@@ -13445,7 +13448,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>5</v>
@@ -13474,7 +13477,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>4</v>
@@ -13503,7 +13506,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>4</v>
@@ -13535,7 +13538,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>2</v>
@@ -13567,7 +13570,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>5</v>
@@ -15269,12 +15272,8 @@
       <c r="I15" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="J15" s="12" t="n">
-        <v>17</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>20</v>
-      </c>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
@@ -15304,9 +15303,7 @@
       <c r="I16" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="K16" s="12" t="n">
-        <v>42</v>
-      </c>
+      <c r="K16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
@@ -15336,9 +15333,7 @@
       <c r="I17" s="7" t="n">
         <v>36</v>
       </c>
-      <c r="K17" s="13" t="n">
-        <v>55</v>
-      </c>
+      <c r="K17" s="13"/>
       <c r="L17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -15859,7 +15854,7 @@
         <v>8</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F38" s="11" t="n">
         <v>27</v>
@@ -16033,11 +16028,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="16.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="14.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="15" width="17.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="15.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="15" width="16.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="15" width="9.18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="15" width="11.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="15" width="14.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="15" width="17.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="15" width="9.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="15" width="6.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="15" width="7.62"/>
@@ -16211,8 +16206,24 @@
       <c r="B15" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
+      <c r="C15" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>0.33</v>
+      </c>
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
     </row>
@@ -16223,8 +16234,24 @@
       <c r="B16" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
+      <c r="C16" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H16" s="15" t="n">
+        <v>0.5</v>
+      </c>
       <c r="K16" s="18"/>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16234,8 +16261,24 @@
       <c r="B17" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
+      <c r="C17" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H17" s="15" t="n">
+        <v>0.5</v>
+      </c>
       <c r="K17" s="19"/>
       <c r="L17" s="19"/>
     </row>
@@ -16373,8 +16416,24 @@
       <c r="B35" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
+      <c r="C35" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F35" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H35" s="15" t="n">
+        <v>0.66</v>
+      </c>
       <c r="J35" s="18"/>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16384,8 +16443,24 @@
       <c r="B36" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
+      <c r="C36" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H36" s="15" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J36" s="18"/>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16395,8 +16470,24 @@
       <c r="B37" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F37" s="18"/>
-      <c r="G37" s="18"/>
+      <c r="C37" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H37" s="15" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J37" s="18"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16406,8 +16497,24 @@
       <c r="B38" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
+      <c r="C38" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J38" s="18"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -16481,7 +16588,7 @@
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="13.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="16.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="23.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="20.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="7" width="7.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="7" width="7.81"/>
@@ -16515,10 +16622,10 @@
         <v>1</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="J1" s="10" t="s">
         <v>52</v>
@@ -16541,13 +16648,13 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>0</v>
@@ -16565,7 +16672,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J2" s="7" t="n">
         <v>8</v>
@@ -16573,13 +16680,13 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>1</v>
@@ -16597,7 +16704,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>14</v>
@@ -16605,13 +16712,13 @@
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>118</v>
-      </c>
       <c r="C4" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>2</v>
@@ -16629,7 +16736,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>22</v>
@@ -16640,13 +16747,13 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>123</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>119</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>4</v>
@@ -16664,7 +16771,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>18</v>
@@ -16675,13 +16782,13 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>8</v>
@@ -16699,7 +16806,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>20</v>
@@ -16710,13 +16817,13 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>0</v>
@@ -16734,7 +16841,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>7</v>
@@ -16742,13 +16849,13 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>2</v>
@@ -16766,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>15</v>
@@ -16777,13 +16884,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>3</v>
@@ -16801,7 +16908,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J9" s="7" t="n">
         <v>17</v>
@@ -16815,13 +16922,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>6</v>
@@ -16839,7 +16946,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>24</v>
@@ -16853,13 +16960,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>8</v>
@@ -16877,7 +16984,7 @@
         <v>2</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>25</v>
@@ -16891,13 +16998,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>1</v>
@@ -16915,7 +17022,7 @@
         <v>2</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>9</v>
@@ -16923,13 +17030,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>3</v>
@@ -16947,7 +17054,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>13</v>
@@ -16958,13 +17065,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>6</v>
@@ -16982,7 +17089,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>25</v>
@@ -16996,13 +17103,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>5</v>
@@ -17020,7 +17127,7 @@
         <v>2</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>20</v>
@@ -17037,13 +17144,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>5</v>
@@ -17061,7 +17168,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>12</v>
@@ -17075,13 +17182,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>2</v>
@@ -17099,7 +17206,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>9</v>
@@ -17113,13 +17220,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>2</v>
@@ -17137,7 +17244,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="J18" s="7" t="n">
         <v>10</v>
@@ -17148,13 +17255,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>3</v>
@@ -17172,7 +17279,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="J19" s="7" t="n">
         <v>14</v>
@@ -17183,13 +17290,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>5</v>
@@ -17207,7 +17314,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>18</v>
@@ -17218,13 +17325,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>8</v>
@@ -17242,7 +17349,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>24</v>
@@ -17253,13 +17360,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>0</v>
@@ -17277,7 +17384,7 @@
         <v>1</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>6</v>
@@ -17285,13 +17392,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>1</v>
@@ -17309,7 +17416,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>8</v>
@@ -17317,13 +17424,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>2</v>
@@ -17341,7 +17448,7 @@
         <v>1</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>11</v>
@@ -17355,13 +17462,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>148</v>
-      </c>
       <c r="C25" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>2</v>
@@ -17379,7 +17486,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>15</v>
@@ -17390,13 +17497,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D26" s="7" t="n">
         <v>3</v>
@@ -17414,7 +17521,7 @@
         <v>2</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="J26" s="7" t="n">
         <v>16</v>
@@ -17428,13 +17535,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>5</v>
@@ -17452,7 +17559,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J27" s="7" t="n">
         <v>18</v>
@@ -17463,13 +17570,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>5</v>
@@ -17487,7 +17594,7 @@
         <v>1</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>21</v>
@@ -17501,13 +17608,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>6</v>
@@ -17525,7 +17632,7 @@
         <v>2</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>19</v>
@@ -17539,13 +17646,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>7</v>
@@ -17563,7 +17670,7 @@
         <v>2</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>18</v>
@@ -17577,13 +17684,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>8</v>
@@ -17601,7 +17708,7 @@
         <v>2</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J31" s="7" t="n">
         <v>23</v>
@@ -17615,13 +17722,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>9</v>
@@ -17639,7 +17746,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="J32" s="7" t="n">
         <v>28</v>
@@ -17653,13 +17760,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>9</v>
@@ -17677,7 +17784,7 @@
         <v>1</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J33" s="7" t="n">
         <v>40</v>
@@ -17688,13 +17795,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>3</v>
@@ -17712,7 +17819,7 @@
         <v>1</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J34" s="7" t="n">
         <v>16</v>
@@ -17723,13 +17830,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>5</v>
@@ -17747,7 +17854,7 @@
         <v>1</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J35" s="7" t="n">
         <v>19</v>
@@ -17758,13 +17865,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D36" s="7" t="n">
         <v>8</v>
@@ -17782,7 +17889,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J36" s="7" t="n">
         <v>24</v>
@@ -17793,10 +17900,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>112</v>
@@ -17817,7 +17924,7 @@
         <v>1</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J37" s="7" t="n">
         <v>15</v>
@@ -17828,10 +17935,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>112</v>
@@ -17852,7 +17959,7 @@
         <v>1</v>
       </c>
       <c r="I38" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J38" s="7" t="n">
         <v>16</v>
@@ -17866,10 +17973,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C39" s="7" t="s">
         <v>112</v>
@@ -17890,7 +17997,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J39" s="7" t="n">
         <v>26</v>
@@ -17904,10 +18011,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B40" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>169</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>112</v>
@@ -17928,7 +18035,7 @@
         <v>1</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="J40" s="7" t="n">
         <v>25</v>
@@ -17942,10 +18049,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>112</v>
@@ -17966,7 +18073,7 @@
         <v>1</v>
       </c>
       <c r="I41" s="7" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="J41" s="7" t="n">
         <v>11</v>
@@ -18032,7 +18139,7 @@
         <v>50</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>52</v>
@@ -18055,10 +18162,10 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>0</v>
@@ -18073,7 +18180,7 @@
         <v>2</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>8</v>
@@ -18081,10 +18188,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>1</v>
@@ -18099,7 +18206,7 @@
         <v>5</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>16</v>
@@ -18107,10 +18214,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>2</v>
@@ -18125,7 +18232,7 @@
         <v>14</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>22</v>
@@ -18133,10 +18240,10 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>3</v>
@@ -18151,7 +18258,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>18</v>
@@ -18159,10 +18266,10 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>4</v>
@@ -18177,7 +18284,7 @@
         <v>19</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>20</v>
@@ -18185,10 +18292,10 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>5</v>
@@ -18203,7 +18310,7 @@
         <v>18</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>18</v>
@@ -18211,10 +18318,10 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>5</v>
@@ -18229,7 +18336,7 @@
         <v>15</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>15</v>
@@ -18237,10 +18344,10 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>6</v>
@@ -18255,7 +18362,7 @@
         <v>23</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>24</v>
@@ -18263,10 +18370,10 @@
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>7</v>
@@ -18281,7 +18388,7 @@
         <v>28</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>25</v>
@@ -18289,10 +18396,10 @@
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>8</v>
@@ -18307,7 +18414,7 @@
         <v>24</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>28</v>
@@ -18315,10 +18422,10 @@
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>8</v>
@@ -18333,7 +18440,7 @@
         <v>28</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>28</v>
@@ -18401,13 +18508,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>3</v>
@@ -18418,13 +18525,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>3</v>
@@ -18475,57 +18582,57 @@
         <v>46</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="N1" s="10" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="O1" s="10" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P1" s="10" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="Q1" s="10" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>5</v>
@@ -18560,7 +18667,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D3" s="7" t="n">
         <v>5</v>
@@ -18598,7 +18705,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>5</v>
@@ -18963,7 +19070,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>5</v>
@@ -19001,7 +19108,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
about to try to move goal performance checker to a place each combatant can have their own
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="240">
   <si>
     <t xml:space="preserve">minDmg</t>
   </si>
@@ -15772,9 +15772,7 @@
       <c r="I35" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="J35" s="11" t="n">
-        <v>18</v>
-      </c>
+      <c r="J35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
@@ -15804,9 +15802,7 @@
       <c r="I36" s="7" t="n">
         <v>24</v>
       </c>
-      <c r="J36" s="11" t="n">
-        <v>35</v>
-      </c>
+      <c r="J36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
@@ -15836,9 +15832,7 @@
       <c r="I37" s="7" t="n">
         <v>34</v>
       </c>
-      <c r="J37" s="11" t="n">
-        <v>50</v>
-      </c>
+      <c r="J37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
@@ -15868,9 +15862,7 @@
       <c r="I38" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="J38" s="11" t="n">
-        <v>60</v>
-      </c>
+      <c r="J38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16290,6 +16282,24 @@
       <c r="B19" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="C19" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H19" s="15" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
@@ -16298,6 +16308,24 @@
       <c r="B20" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="C20" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G20" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <v>0.33</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
@@ -16306,6 +16334,24 @@
       <c r="B21" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="C21" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
@@ -16313,6 +16359,24 @@
       </c>
       <c r="B22" s="7" t="s">
         <v>67</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -16525,6 +16589,24 @@
       <c r="B40" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="C40" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
@@ -16533,6 +16615,24 @@
       <c r="B41" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="C41" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F41" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H41" s="15" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
@@ -16541,6 +16641,24 @@
       <c r="B42" s="7" t="s">
         <v>67</v>
       </c>
+      <c r="C42" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H42" s="15" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
@@ -16548,6 +16666,24 @@
       </c>
       <c r="B43" s="7" t="s">
         <v>67</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F43" s="18" t="s">
+        <v>114</v>
+      </c>
+      <c r="G43" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="H43" s="15" t="n">
+        <v>0.75</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
armor class studies added
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1237" uniqueCount="237">
   <si>
     <t xml:space="preserve">Total AC Body+Headgear per tier</t>
   </si>
@@ -458,6 +458,42 @@
     <t xml:space="preserve">EtherBow</t>
   </si>
   <si>
+    <t xml:space="preserve">PotLid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buckler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LanternShield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AncientBuckler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CabinetDoor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aspis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KiteShield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GothicShield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pavise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TowerShield</t>
+  </si>
+  <si>
     <t xml:space="preserve">affixProfile</t>
   </si>
   <si>
@@ -575,49 +611,13 @@
     <t xml:space="preserve">shieldSize</t>
   </si>
   <si>
-    <t xml:space="preserve">PotLid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shield</t>
-  </si>
-  <si>
     <t xml:space="preserve">Small</t>
   </si>
   <si>
-    <t xml:space="preserve">CabinetDoor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heater</t>
-  </si>
-  <si>
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
-    <t xml:space="preserve">Buckler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pavise</t>
-  </si>
-  <si>
     <t xml:space="preserve">Large</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aspis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LanternShield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KiteShield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TowerShield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AncientBuckler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GothicShield</t>
   </si>
   <si>
     <t xml:space="preserve">Ring</t>
@@ -4890,6 +4890,360 @@
         <v>0.25</v>
       </c>
     </row>
+    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G100" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H100" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I100" s="5" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D101" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F101" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G101" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H101" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I101" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G102" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="H102" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I102" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="0"/>
+      <c r="C103" s="2"/>
+    </row>
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E104" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G104" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H104" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I104" s="5" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C105" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D105" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E105" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G105" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H105" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I105" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C106" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E106" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F106" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G106" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H106" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I106" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C107" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D107" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E107" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F107" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G107" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H107" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I107" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C108" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D108" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E108" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F108" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G108" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H108" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I108" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="0"/>
+      <c r="C109" s="2"/>
+    </row>
+    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E110" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F110" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="G110" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H110" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I110" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C111" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D111" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E111" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F111" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="G111" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H111" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I111" s="5" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="0"/>
+    </row>
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="0"/>
+    </row>
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="0"/>
+    </row>
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D118" s="0"/>
+    </row>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D119" s="0"/>
+    </row>
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D120" s="0"/>
+    </row>
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D121" s="0"/>
+    </row>
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D122" s="0"/>
+    </row>
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D123" s="0"/>
+    </row>
+    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D124" s="0"/>
+    </row>
+    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D125" s="0"/>
+    </row>
+    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D126" s="0"/>
+    </row>
+    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D127" s="0"/>
+    </row>
+    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D128" s="0"/>
+    </row>
+    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D129" s="0"/>
+    </row>
+    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D130" s="0"/>
+    </row>
+    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D131" s="0"/>
+    </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -4936,40 +5290,40 @@
         <v>33</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4980,7 +5334,7 @@
         <v>42</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>1</v>
@@ -5009,7 +5363,7 @@
         <v>42</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>2</v>
@@ -5039,7 +5393,7 @@
         <v>42</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>3</v>
@@ -5069,7 +5423,7 @@
         <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>6</v>
@@ -5099,7 +5453,7 @@
         <v>42</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>8</v>
@@ -5130,7 +5484,7 @@
         <v>53</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>1</v>
@@ -5159,7 +5513,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>2</v>
@@ -5188,7 +5542,7 @@
         <v>53</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>3</v>
@@ -5217,7 +5571,7 @@
         <v>53</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>5</v>
@@ -5246,7 +5600,7 @@
         <v>53</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>7</v>
@@ -5276,7 +5630,7 @@
         <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>3</v>
@@ -5307,7 +5661,7 @@
         <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>5</v>
@@ -5338,7 +5692,7 @@
         <v>42</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>6</v>
@@ -5369,7 +5723,7 @@
         <v>42</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>8</v>
@@ -5402,7 +5756,7 @@
         <v>53</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>1</v>
@@ -5431,7 +5785,7 @@
         <v>53</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>3</v>
@@ -5460,7 +5814,7 @@
         <v>53</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>4</v>
@@ -5489,7 +5843,7 @@
         <v>53</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>9</v>
@@ -5519,7 +5873,7 @@
         <v>42</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>3</v>
@@ -5550,7 +5904,7 @@
         <v>42</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>4</v>
@@ -5581,7 +5935,7 @@
         <v>42</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>5</v>
@@ -5611,7 +5965,7 @@
         <v>42</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>6</v>
@@ -5642,7 +5996,7 @@
         <v>42</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>8</v>
@@ -5675,7 +6029,7 @@
         <v>53</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>3</v>
@@ -5704,7 +6058,7 @@
         <v>53</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>4</v>
@@ -5733,7 +6087,7 @@
         <v>53</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>5</v>
@@ -5762,7 +6116,7 @@
         <v>53</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D33" s="2" t="n">
         <v>7</v>
@@ -5792,7 +6146,7 @@
         <v>42</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>2</v>
@@ -5822,7 +6176,7 @@
         <v>42</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>4</v>
@@ -5852,7 +6206,7 @@
         <v>42</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="D37" s="2" t="n">
         <v>5</v>
@@ -5882,7 +6236,7 @@
         <v>42</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="D38" s="2" t="n">
         <v>8</v>
@@ -5913,7 +6267,7 @@
         <v>53</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>2</v>
@@ -5942,7 +6296,7 @@
         <v>53</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>4</v>
@@ -5971,7 +6325,7 @@
         <v>53</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>6</v>
@@ -6000,7 +6354,7 @@
         <v>53</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="D43" s="2" t="n">
         <v>9</v>
@@ -6077,43 +6431,43 @@
         <v>33</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6124,7 +6478,7 @@
         <v>92</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0</v>
@@ -6142,7 +6496,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>8</v>
@@ -6156,7 +6510,7 @@
         <v>92</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>1</v>
@@ -6174,7 +6528,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>14</v>
@@ -6188,7 +6542,7 @@
         <v>92</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>2</v>
@@ -6206,7 +6560,7 @@
         <v>1</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>22</v>
@@ -6223,7 +6577,7 @@
         <v>92</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>4</v>
@@ -6241,7 +6595,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>18</v>
@@ -6258,7 +6612,7 @@
         <v>92</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>8</v>
@@ -6276,7 +6630,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>20</v>
@@ -6293,7 +6647,7 @@
         <v>92</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0</v>
@@ -6311,7 +6665,7 @@
         <v>1</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>7</v>
@@ -6325,7 +6679,7 @@
         <v>92</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>2</v>
@@ -6343,7 +6697,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>15</v>
@@ -6360,7 +6714,7 @@
         <v>92</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>3</v>
@@ -6378,7 +6732,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>17</v>
@@ -6398,7 +6752,7 @@
         <v>92</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>6</v>
@@ -6416,7 +6770,7 @@
         <v>1</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>24</v>
@@ -6436,7 +6790,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>8</v>
@@ -6454,7 +6808,7 @@
         <v>2</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>25</v>
@@ -6474,7 +6828,7 @@
         <v>92</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
@@ -6492,7 +6846,7 @@
         <v>2</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>9</v>
@@ -6506,7 +6860,7 @@
         <v>92</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>3</v>
@@ -6524,7 +6878,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>13</v>
@@ -6541,7 +6895,7 @@
         <v>92</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>6</v>
@@ -6559,7 +6913,7 @@
         <v>1</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>25</v>
@@ -6579,7 +6933,7 @@
         <v>92</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>5</v>
@@ -6597,7 +6951,7 @@
         <v>2</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>20</v>
@@ -6620,7 +6974,7 @@
         <v>92</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>5</v>
@@ -6638,7 +6992,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>12</v>
@@ -6658,7 +7012,7 @@
         <v>92</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>2</v>
@@ -6676,7 +7030,7 @@
         <v>1</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>9</v>
@@ -6696,7 +7050,7 @@
         <v>92</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>2</v>
@@ -6714,7 +7068,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>10</v>
@@ -6731,7 +7085,7 @@
         <v>92</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>3</v>
@@ -6749,7 +7103,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>14</v>
@@ -6766,7 +7120,7 @@
         <v>92</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>5</v>
@@ -6784,7 +7138,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>18</v>
@@ -6801,7 +7155,7 @@
         <v>92</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>8</v>
@@ -6819,7 +7173,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>24</v>
@@ -6854,7 +7208,7 @@
         <v>1</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>6</v>
@@ -6886,7 +7240,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>8</v>
@@ -6918,7 +7272,7 @@
         <v>1</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>11</v>
@@ -6956,7 +7310,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>15</v>
@@ -6991,7 +7345,7 @@
         <v>2</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>16</v>
@@ -7029,7 +7383,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>18</v>
@@ -7064,7 +7418,7 @@
         <v>1</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>21</v>
@@ -7102,7 +7456,7 @@
         <v>2</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>19</v>
@@ -7140,7 +7494,7 @@
         <v>2</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>18</v>
@@ -7178,7 +7532,7 @@
         <v>2</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>23</v>
@@ -7216,7 +7570,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>28</v>
@@ -7254,7 +7608,7 @@
         <v>1</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>40</v>
@@ -7271,7 +7625,7 @@
         <v>117</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>3</v>
@@ -7289,7 +7643,7 @@
         <v>1</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>16</v>
@@ -7306,7 +7660,7 @@
         <v>117</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>5</v>
@@ -7324,7 +7678,7 @@
         <v>1</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>19</v>
@@ -7341,7 +7695,7 @@
         <v>117</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>8</v>
@@ -7359,7 +7713,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>24</v>
@@ -7394,7 +7748,7 @@
         <v>1</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>15</v>
@@ -7429,7 +7783,7 @@
         <v>1</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>16</v>
@@ -7467,7 +7821,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>26</v>
@@ -7505,7 +7859,7 @@
         <v>1</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>25</v>
@@ -7543,7 +7897,7 @@
         <v>1</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>11</v>
@@ -7594,48 +7948,48 @@
         <v>32</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>0</v>
@@ -7650,7 +8004,7 @@
         <v>2</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>8</v>
@@ -7658,10 +8012,10 @@
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>180</v>
+        <v>143</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>1</v>
@@ -7676,7 +8030,7 @@
         <v>5</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>16</v>
@@ -7684,10 +8038,10 @@
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>181</v>
+        <v>144</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>2</v>
@@ -7702,7 +8056,7 @@
         <v>14</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>22</v>
@@ -7710,10 +8064,10 @@
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>183</v>
+        <v>139</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>3</v>
@@ -7728,7 +8082,7 @@
         <v>13</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>18</v>
@@ -7736,10 +8090,10 @@
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>184</v>
+        <v>148</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>4</v>
@@ -7754,7 +8108,7 @@
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>20</v>
@@ -7762,10 +8116,10 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>186</v>
+        <v>145</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>5</v>
@@ -7780,7 +8134,7 @@
         <v>18</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>18</v>
@@ -7788,10 +8142,10 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>187</v>
+        <v>141</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>5</v>
@@ -7806,7 +8160,7 @@
         <v>15</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>15</v>
@@ -7814,10 +8168,10 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>188</v>
+        <v>146</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C9" s="2" t="n">
         <v>6</v>
@@ -7832,7 +8186,7 @@
         <v>23</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>24</v>
@@ -7840,10 +8194,10 @@
     </row>
     <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>189</v>
+        <v>149</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C10" s="2" t="n">
         <v>7</v>
@@ -7858,7 +8212,7 @@
         <v>28</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>25</v>
@@ -7866,10 +8220,10 @@
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>190</v>
+        <v>142</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C11" s="2" t="n">
         <v>8</v>
@@ -7884,7 +8238,7 @@
         <v>24</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>28</v>
@@ -7892,10 +8246,10 @@
     </row>
     <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>191</v>
+        <v>147</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="C12" s="2" t="n">
         <v>8</v>
@@ -7910,7 +8264,7 @@
         <v>28</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>28</v>
@@ -7949,31 +8303,31 @@
         <v>33</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8049,7 +8403,7 @@
   <sheetData>
     <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>195</v>
@@ -8102,7 +8456,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>5</v>
@@ -8175,7 +8529,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>5</v>
@@ -8239,7 +8593,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>5</v>
@@ -8277,7 +8631,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>3</v>
@@ -8315,7 +8669,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>5</v>
@@ -8353,7 +8707,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>3</v>
@@ -8385,7 +8739,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>5</v>
@@ -8423,7 +8777,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>3</v>
@@ -8464,7 +8818,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>5</v>
@@ -8505,7 +8859,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>3</v>
@@ -8540,7 +8894,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>178</v>
+        <v>140</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>5</v>
@@ -8654,7 +9008,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>187</v>
+        <v>141</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>213</v>

</xml_diff>

<commit_message>
added speed enjoyer study
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="balancing" sheetId="1" state="visible" r:id="rId2"/>
@@ -4394,7 +4394,7 @@
         <v>48</v>
       </c>
       <c r="I78" s="5" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6408,7 +6408,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr defaultColWidth="8.43359375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="13.87"/>
@@ -6635,9 +6635,6 @@
       <c r="J6" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="K6" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -6702,9 +6699,6 @@
       <c r="J8" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="K8" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -6737,12 +6731,6 @@
       <c r="J9" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="K9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L9" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
@@ -6775,12 +6763,6 @@
       <c r="J10" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="K10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
@@ -6813,12 +6795,6 @@
       <c r="J11" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -6883,9 +6859,6 @@
       <c r="J13" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="L13" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
@@ -6918,12 +6891,6 @@
       <c r="J14" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L14" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
@@ -6956,15 +6923,6 @@
       <c r="J15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="K15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
@@ -6997,12 +6955,6 @@
       <c r="J16" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="K16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M16" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
@@ -7035,12 +6987,6 @@
       <c r="J17" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="K17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
@@ -7073,9 +7019,6 @@
       <c r="J18" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="M18" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
@@ -7108,9 +7051,6 @@
       <c r="J19" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="M19" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
@@ -7143,9 +7083,6 @@
       <c r="J20" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="M20" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
@@ -7178,9 +7115,6 @@
       <c r="J21" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="M21" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
@@ -7260,7 +7194,7 @@
         <v>2</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>3</v>
@@ -7276,12 +7210,6 @@
       </c>
       <c r="J24" s="2" t="n">
         <v>11</v>
-      </c>
-      <c r="K24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7298,7 +7226,7 @@
         <v>2</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>1</v>
@@ -7314,9 +7242,6 @@
       </c>
       <c r="J25" s="2" t="n">
         <v>15</v>
-      </c>
-      <c r="K25" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7330,7 +7255,7 @@
         <v>73</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>6</v>
@@ -7349,12 +7274,6 @@
       </c>
       <c r="J26" s="2" t="n">
         <v>16</v>
-      </c>
-      <c r="K26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L26" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7388,9 +7307,6 @@
       <c r="J27" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="K27" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
@@ -7423,12 +7339,6 @@
       <c r="J28" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="K28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L28" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
@@ -7461,12 +7371,6 @@
       <c r="J29" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="K29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
@@ -7499,12 +7403,6 @@
       <c r="J30" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="K30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
@@ -7537,12 +7435,6 @@
       <c r="J31" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="K31" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M31" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
@@ -7575,12 +7467,6 @@
       <c r="J32" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L32" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
@@ -7613,9 +7499,6 @@
       <c r="J33" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="K33" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
@@ -7648,9 +7531,6 @@
       <c r="J34" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="M34" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
@@ -7683,9 +7563,6 @@
       <c r="J35" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="M35" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
@@ -7718,9 +7595,6 @@
       <c r="J36" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="M36" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
@@ -7753,9 +7627,6 @@
       <c r="J37" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="L37" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
@@ -7788,12 +7659,6 @@
       <c r="J38" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="K38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L38" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
@@ -7826,12 +7691,6 @@
       <c r="J39" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="K39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L39" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
@@ -7864,12 +7723,6 @@
       <c r="J40" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K40" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L40" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
@@ -7902,13 +7755,22 @@
       <c r="J41" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="L41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M41" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
deploy for job interview
</commit_message>
<xml_diff>
--- a/packages/balance-tools/game-data.xlsx
+++ b/packages/balance-tools/game-data.xlsx
@@ -762,7 +762,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -797,12 +797,6 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -853,7 +847,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -874,27 +868,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1730,44 +1704,44 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>223</v>
       </c>
     </row>
@@ -1877,44 +1851,44 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>223</v>
       </c>
     </row>
@@ -2240,44 +2214,44 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>223</v>
       </c>
     </row>
@@ -2611,26 +2585,26 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="16.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="17.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="5" width="15.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="5" width="16.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="5" width="9.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="5" width="11.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="5" width="17.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="5" width="9.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="5" width="6.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="5" width="7.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="5" width="7.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="5" width="6.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="5" width="7.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="17.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="15.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="9.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="17.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="9.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="6.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="7.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="7.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="6.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="7.11"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="11.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C1" s="2" t="s">
@@ -2639,28 +2613,28 @@
       <c r="D1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="6"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -2669,8 +2643,8 @@
       <c r="B2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -2679,29 +2653,29 @@
       <c r="B3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="I3" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="M3" s="9"/>
-      <c r="P3" s="0"/>
+      <c r="M3" s="6"/>
+      <c r="P3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -2710,28 +2684,28 @@
       <c r="B4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="M4" s="9"/>
+      <c r="M4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -2740,28 +2714,28 @@
       <c r="B5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="M5" s="9"/>
+      <c r="M5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -2770,28 +2744,28 @@
       <c r="B6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="M6" s="9"/>
+      <c r="M6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2809,25 +2783,25 @@
       <c r="B9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I9" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -2838,25 +2812,25 @@
       <c r="B10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -2867,25 +2841,25 @@
       <c r="B11" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -2896,25 +2870,25 @@
       <c r="B12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="2" t="n">
         <v>0.66</v>
       </c>
     </row>
@@ -2926,28 +2900,28 @@
       <c r="B14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="L14" s="9"/>
+      <c r="L14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
@@ -2956,29 +2930,29 @@
       <c r="B15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I15" s="2" t="n">
         <v>0.4</v>
       </c>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
@@ -2987,28 +2961,28 @@
       <c r="B16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="L16" s="9"/>
+      <c r="L16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
@@ -3017,29 +2991,29 @@
       <c r="B17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I17" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3049,26 +3023,26 @@
       <c r="B19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="5" t="n">
-        <v>0.5</v>
+      <c r="I19" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3078,25 +3052,25 @@
       <c r="B20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="2" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -3107,25 +3081,25 @@
       <c r="B21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I21" s="5" t="n">
+      <c r="I21" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -3136,25 +3110,25 @@
       <c r="B22" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="G22" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="I22" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -3166,29 +3140,29 @@
       <c r="B24" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="9" t="s">
+      <c r="G24" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="H24" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="9"/>
-      <c r="M24" s="9"/>
+      <c r="K24" s="6"/>
+      <c r="M24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
@@ -3197,29 +3171,29 @@
       <c r="B25" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G25" s="9" t="s">
+      <c r="G25" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="H25" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I25" s="5" t="n">
+      <c r="I25" s="2" t="n">
         <v>0.25</v>
       </c>
-      <c r="K25" s="9"/>
-      <c r="M25" s="9"/>
+      <c r="K25" s="6"/>
+      <c r="M25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
@@ -3228,29 +3202,29 @@
       <c r="B26" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G26" s="9" t="s">
+      <c r="G26" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="2" t="n">
         <v>0.33</v>
       </c>
-      <c r="K26" s="9"/>
-      <c r="M26" s="9"/>
+      <c r="K26" s="6"/>
+      <c r="M26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
@@ -3259,29 +3233,29 @@
       <c r="B27" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H27" s="5" t="s">
+      <c r="H27" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I27" s="5" t="n">
+      <c r="I27" s="2" t="n">
         <v>0.25</v>
       </c>
-      <c r="K27" s="9"/>
-      <c r="L27" s="9"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
@@ -3290,28 +3264,28 @@
       <c r="B28" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="F28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G28" s="9" t="s">
+      <c r="G28" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="H28" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I28" s="5" t="n">
+      <c r="I28" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="L28" s="9"/>
+      <c r="L28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
@@ -3320,28 +3294,28 @@
       <c r="B29" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G29" s="9" t="s">
+      <c r="G29" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="H29" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I29" s="5" t="n">
+      <c r="I29" s="2" t="n">
         <v>0.66</v>
       </c>
-      <c r="L29" s="9"/>
+      <c r="L29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
@@ -3350,29 +3324,29 @@
       <c r="B30" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="9" t="s">
+      <c r="G30" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="2" t="n">
         <v>0.66</v>
       </c>
-      <c r="L30" s="9"/>
-      <c r="M30" s="9"/>
+      <c r="L30" s="6"/>
+      <c r="M30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
@@ -3381,29 +3355,29 @@
       <c r="B31" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E31" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="F31" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G31" s="9" t="s">
+      <c r="G31" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="H31" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I31" s="5" t="n">
+      <c r="I31" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3421,25 +3395,25 @@
       <c r="B34" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="9" t="s">
+      <c r="G34" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I34" s="5" t="n">
+      <c r="I34" s="2" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -3450,25 +3424,25 @@
       <c r="B35" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E35" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F35" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="G35" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="H35" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I35" s="5" t="n">
+      <c r="I35" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -3479,25 +3453,25 @@
       <c r="B36" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="E36" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F36" s="5" t="s">
+      <c r="F36" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="9" t="s">
+      <c r="G36" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H36" s="9" t="s">
+      <c r="H36" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I36" s="5" t="n">
+      <c r="I36" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -3508,25 +3482,25 @@
       <c r="B37" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="5" t="s">
+      <c r="F37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I37" s="5" t="n">
+      <c r="I37" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -3538,28 +3512,28 @@
       <c r="B39" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="F39" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G39" s="9" t="s">
+      <c r="G39" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="H39" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I39" s="5" t="n">
+      <c r="I39" s="2" t="n">
         <v>0.66</v>
       </c>
-      <c r="K39" s="9"/>
+      <c r="K39" s="6"/>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
@@ -3568,28 +3542,28 @@
       <c r="B40" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E40" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G40" s="9" t="s">
+      <c r="G40" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="H40" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I40" s="5" t="n">
+      <c r="I40" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="K40" s="9"/>
+      <c r="K40" s="6"/>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
@@ -3598,28 +3572,28 @@
       <c r="B41" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D41" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E41" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="G41" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="H41" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I41" s="2" t="n">
         <v>0.75</v>
       </c>
-      <c r="K41" s="9"/>
+      <c r="K41" s="6"/>
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
@@ -3628,28 +3602,28 @@
       <c r="B42" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="D42" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G42" s="9" t="s">
+      <c r="G42" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H42" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I42" s="5" t="n">
+      <c r="I42" s="2" t="n">
         <v>0.75</v>
       </c>
-      <c r="K42" s="9"/>
+      <c r="K42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3659,25 +3633,25 @@
       <c r="B44" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="D44" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="E44" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F44" s="5" t="s">
+      <c r="F44" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G44" s="9" t="s">
+      <c r="G44" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I44" s="5" t="n">
+      <c r="I44" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3688,25 +3662,25 @@
       <c r="B45" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="D45" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="E45" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G45" s="9" t="s">
+      <c r="G45" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I45" s="5" t="n">
+      <c r="I45" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -3717,25 +3691,25 @@
       <c r="B46" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="D46" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="E46" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G46" s="9" t="s">
+      <c r="G46" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="H46" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I46" s="5" t="n">
+      <c r="I46" s="2" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -3746,25 +3720,25 @@
       <c r="B47" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="D47" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E47" s="5" t="s">
+      <c r="E47" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="F47" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G47" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="H47" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I47" s="5" t="n">
+      <c r="I47" s="2" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -3784,26 +3758,26 @@
       <c r="B50" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="D50" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="E50" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="F50" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H50" s="9" t="s">
+      <c r="H50" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I50" s="5" t="n">
-        <v>0.5</v>
+      <c r="I50" s="2" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3813,25 +3787,25 @@
       <c r="B51" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="D51" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="E51" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="F51" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H51" s="9" t="s">
+      <c r="H51" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I51" s="5" t="n">
+      <c r="I51" s="2" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -3842,25 +3816,25 @@
       <c r="B52" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="D52" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E52" s="5" t="s">
+      <c r="E52" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F52" s="5" t="s">
+      <c r="F52" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G52" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H52" s="9" t="s">
+      <c r="H52" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I52" s="5" t="n">
+      <c r="I52" s="2" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -3871,25 +3845,25 @@
       <c r="B53" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="D53" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E53" s="5" t="s">
+      <c r="E53" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F53" s="5" t="s">
+      <c r="F53" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="G53" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H53" s="9" t="s">
+      <c r="H53" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I53" s="5" t="n">
+      <c r="I53" s="2" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -3901,8 +3875,8 @@
       <c r="B55" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G55" s="9"/>
-      <c r="H55" s="9"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
@@ -3911,25 +3885,25 @@
       <c r="B56" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="C56" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="5" t="s">
+      <c r="D56" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E56" s="5" t="s">
+      <c r="E56" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F56" s="5" t="s">
+      <c r="F56" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G56" s="9" t="s">
+      <c r="G56" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H56" s="9" t="s">
+      <c r="H56" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I56" s="5" t="n">
+      <c r="I56" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3940,25 +3914,25 @@
       <c r="B57" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C57" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D57" s="5" t="s">
+      <c r="D57" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E57" s="5" t="s">
+      <c r="E57" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F57" s="5" t="s">
+      <c r="F57" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G57" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H57" s="9" t="s">
+      <c r="H57" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I57" s="5" t="n">
+      <c r="I57" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3969,25 +3943,25 @@
       <c r="B58" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D58" s="5" t="s">
+      <c r="D58" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E58" s="5" t="s">
+      <c r="E58" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F58" s="5" t="s">
+      <c r="F58" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G58" s="9" t="s">
+      <c r="G58" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="H58" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I58" s="5" t="n">
+      <c r="I58" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3999,25 +3973,25 @@
       <c r="B60" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D60" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E60" s="5" t="s">
+      <c r="E60" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F60" s="5" t="s">
+      <c r="F60" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G60" s="9" t="s">
+      <c r="G60" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H60" s="9" t="s">
+      <c r="H60" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I60" s="5" t="n">
+      <c r="I60" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -4028,45 +4002,45 @@
       <c r="B61" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C61" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D61" s="5" t="s">
+      <c r="D61" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="E61" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F61" s="5" t="s">
+      <c r="F61" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G61" s="9" t="s">
+      <c r="G61" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H61" s="9" t="s">
+      <c r="H61" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I61" s="5" t="n">
-        <v>0.5</v>
+      <c r="I61" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0"/>
-      <c r="B62" s="0"/>
-      <c r="C62" s="0"/>
-      <c r="D62" s="0"/>
-      <c r="E62" s="0"/>
-      <c r="F62" s="0"/>
-      <c r="G62" s="0"/>
-      <c r="H62" s="0"/>
-      <c r="I62" s="0"/>
-      <c r="J62" s="0"/>
-      <c r="K62" s="0"/>
-      <c r="L62" s="0"/>
-      <c r="M62" s="0"/>
-      <c r="N62" s="0"/>
-      <c r="O62" s="0"/>
-      <c r="P62" s="0"/>
+      <c r="A62" s="7"/>
+      <c r="B62" s="7"/>
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+      <c r="J62" s="7"/>
+      <c r="K62" s="7"/>
+      <c r="L62" s="7"/>
+      <c r="M62" s="7"/>
+      <c r="N62" s="7"/>
+      <c r="O62" s="7"/>
+      <c r="P62" s="7"/>
     </row>
     <row r="63" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
@@ -4075,25 +4049,25 @@
       <c r="B63" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="C63" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D63" s="5" t="s">
+      <c r="D63" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E63" s="5" t="s">
+      <c r="E63" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F63" s="5" t="s">
+      <c r="F63" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G63" s="9" t="s">
+      <c r="G63" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H63" s="9" t="s">
+      <c r="H63" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I63" s="5" t="n">
+      <c r="I63" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -4104,25 +4078,25 @@
       <c r="B64" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C64" s="5" t="s">
+      <c r="C64" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D64" s="5" t="s">
+      <c r="D64" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E64" s="5" t="s">
+      <c r="E64" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F64" s="5" t="s">
+      <c r="F64" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G64" s="9" t="s">
+      <c r="G64" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H64" s="9" t="s">
+      <c r="H64" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I64" s="5" t="n">
+      <c r="I64" s="2" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -4134,25 +4108,25 @@
       <c r="B66" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="C66" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="E66" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F66" s="5" t="s">
+      <c r="F66" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="G66" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H66" s="5" t="s">
+      <c r="H66" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I66" s="5" t="n">
+      <c r="I66" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4163,25 +4137,25 @@
       <c r="B67" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C67" s="5" t="s">
+      <c r="C67" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D67" s="5" t="s">
+      <c r="D67" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E67" s="5" t="s">
+      <c r="E67" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F67" s="5" t="s">
+      <c r="F67" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G67" s="9" t="s">
+      <c r="G67" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H67" s="5" t="s">
+      <c r="H67" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I67" s="5" t="n">
+      <c r="I67" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4192,25 +4166,25 @@
       <c r="B68" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C68" s="5" t="s">
+      <c r="C68" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D68" s="5" t="s">
+      <c r="D68" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E68" s="5" t="s">
+      <c r="E68" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F68" s="5" t="s">
+      <c r="F68" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G68" s="9" t="s">
+      <c r="G68" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H68" s="5" t="s">
+      <c r="H68" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I68" s="5" t="n">
+      <c r="I68" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4222,25 +4196,25 @@
       <c r="B70" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="D70" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E70" s="5" t="s">
+      <c r="E70" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F70" s="5" t="s">
+      <c r="F70" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G70" s="9" t="s">
+      <c r="G70" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H70" s="5" t="s">
+      <c r="H70" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I70" s="5" t="n">
+      <c r="I70" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4251,25 +4225,25 @@
       <c r="B71" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C71" s="5" t="s">
+      <c r="C71" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D71" s="5" t="s">
+      <c r="D71" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E71" s="5" t="s">
+      <c r="E71" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F71" s="5" t="s">
+      <c r="F71" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G71" s="9" t="s">
+      <c r="G71" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H71" s="5" t="s">
+      <c r="H71" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I71" s="5" t="n">
+      <c r="I71" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4280,25 +4254,25 @@
       <c r="B72" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C72" s="5" t="s">
+      <c r="C72" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D72" s="5" t="s">
+      <c r="D72" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E72" s="5" t="s">
+      <c r="E72" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F72" s="5" t="s">
+      <c r="F72" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G72" s="9" t="s">
+      <c r="G72" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H72" s="5" t="s">
+      <c r="H72" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I72" s="5" t="n">
+      <c r="I72" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4309,25 +4283,25 @@
       <c r="B73" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C73" s="5" t="s">
+      <c r="C73" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D73" s="5" t="s">
+      <c r="D73" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E73" s="5" t="s">
+      <c r="E73" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="F73" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G73" s="9" t="s">
+      <c r="G73" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H73" s="5" t="s">
+      <c r="H73" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I73" s="5" t="n">
+      <c r="I73" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4346,25 +4320,25 @@
       <c r="B76" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C76" s="5" t="s">
+      <c r="C76" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D76" s="5" t="s">
+      <c r="D76" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E76" s="5" t="s">
+      <c r="E76" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F76" s="5" t="s">
+      <c r="F76" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G76" s="9" t="s">
+      <c r="G76" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H76" s="9" t="s">
+      <c r="H76" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I76" s="5" t="n">
+      <c r="I76" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4375,25 +4349,25 @@
       <c r="B78" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C78" s="5" t="s">
+      <c r="C78" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E78" s="5" t="s">
+      <c r="E78" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F78" s="5" t="s">
+      <c r="F78" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G78" s="9" t="s">
+      <c r="G78" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H78" s="9" t="s">
+      <c r="H78" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I78" s="5" t="n">
+      <c r="I78" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4404,25 +4378,25 @@
       <c r="B79" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C79" s="5" t="s">
+      <c r="C79" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D79" s="5" t="s">
+      <c r="D79" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E79" s="5" t="s">
+      <c r="E79" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F79" s="5" t="s">
+      <c r="F79" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G79" s="9" t="s">
+      <c r="G79" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H79" s="9" t="s">
+      <c r="H79" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I79" s="5" t="n">
+      <c r="I79" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4433,25 +4407,25 @@
       <c r="B80" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C80" s="5" t="s">
+      <c r="C80" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D80" s="5" t="s">
+      <c r="D80" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E80" s="5" t="s">
+      <c r="E80" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F80" s="5" t="s">
+      <c r="F80" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G80" s="9" t="s">
+      <c r="G80" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H80" s="9" t="s">
+      <c r="H80" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I80" s="5" t="n">
+      <c r="I80" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4462,25 +4436,25 @@
       <c r="B81" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C81" s="5" t="s">
+      <c r="C81" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D81" s="5" t="s">
+      <c r="D81" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E81" s="5" t="s">
+      <c r="E81" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F81" s="5" t="s">
+      <c r="F81" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G81" s="9" t="s">
+      <c r="G81" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H81" s="9" t="s">
+      <c r="H81" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I81" s="5" t="n">
+      <c r="I81" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4491,25 +4465,25 @@
       <c r="B82" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C82" s="5" t="s">
+      <c r="C82" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E82" s="5" t="s">
+      <c r="E82" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F82" s="5" t="s">
+      <c r="F82" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G82" s="9" t="s">
+      <c r="G82" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H82" s="9" t="s">
+      <c r="H82" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I82" s="5" t="n">
+      <c r="I82" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4520,25 +4494,25 @@
       <c r="B83" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C83" s="5" t="s">
+      <c r="C83" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D83" s="5" t="s">
+      <c r="D83" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E83" s="5" t="s">
+      <c r="E83" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F83" s="5" t="s">
+      <c r="F83" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G83" s="9" t="s">
+      <c r="G83" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H83" s="9" t="s">
+      <c r="H83" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I83" s="5" t="n">
+      <c r="I83" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4549,25 +4523,25 @@
       <c r="B84" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C84" s="5" t="s">
+      <c r="C84" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D84" s="5" t="s">
+      <c r="D84" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E84" s="5" t="s">
+      <c r="E84" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F84" s="5" t="s">
+      <c r="F84" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G84" s="9" t="s">
+      <c r="G84" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H84" s="9" t="s">
+      <c r="H84" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I84" s="5" t="n">
+      <c r="I84" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4578,25 +4552,25 @@
       <c r="B85" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C85" s="5" t="s">
+      <c r="C85" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D85" s="5" t="s">
+      <c r="D85" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E85" s="5" t="s">
+      <c r="E85" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F85" s="5" t="s">
+      <c r="F85" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G85" s="9" t="s">
+      <c r="G85" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H85" s="9" t="s">
+      <c r="H85" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I85" s="5" t="n">
+      <c r="I85" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4607,25 +4581,25 @@
       <c r="B86" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C86" s="5" t="s">
+      <c r="C86" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D86" s="5" t="s">
+      <c r="D86" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E86" s="5" t="s">
+      <c r="E86" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F86" s="5" t="s">
+      <c r="F86" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G86" s="9" t="s">
+      <c r="G86" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H86" s="9" t="s">
+      <c r="H86" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I86" s="5" t="n">
+      <c r="I86" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4636,25 +4610,25 @@
       <c r="B87" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C87" s="5" t="s">
+      <c r="C87" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D87" s="5" t="s">
+      <c r="D87" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E87" s="5" t="s">
+      <c r="E87" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F87" s="5" t="s">
+      <c r="F87" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G87" s="9" t="s">
+      <c r="G87" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H87" s="9" t="s">
+      <c r="H87" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I87" s="5" t="n">
+      <c r="I87" s="2" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -4665,25 +4639,25 @@
       <c r="B89" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C89" s="5" t="s">
+      <c r="C89" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D89" s="5" t="s">
+      <c r="D89" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E89" s="5" t="s">
+      <c r="E89" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F89" s="5" t="s">
+      <c r="F89" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G89" s="9" t="s">
+      <c r="G89" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H89" s="5" t="s">
+      <c r="H89" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I89" s="5" t="n">
+      <c r="I89" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4694,25 +4668,25 @@
       <c r="B90" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C90" s="5" t="s">
+      <c r="C90" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D90" s="5" t="s">
+      <c r="D90" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E90" s="5" t="s">
+      <c r="E90" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F90" s="5" t="s">
+      <c r="F90" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G90" s="9" t="s">
+      <c r="G90" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H90" s="5" t="s">
+      <c r="H90" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I90" s="5" t="n">
+      <c r="I90" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4723,25 +4697,25 @@
       <c r="B91" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C91" s="5" t="s">
+      <c r="C91" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D91" s="5" t="s">
+      <c r="D91" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E91" s="5" t="s">
+      <c r="E91" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F91" s="5" t="s">
+      <c r="F91" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G91" s="9" t="s">
+      <c r="G91" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H91" s="5" t="s">
+      <c r="H91" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I91" s="5" t="n">
+      <c r="I91" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4752,25 +4726,25 @@
       <c r="B93" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C93" s="5" t="s">
+      <c r="C93" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D93" s="5" t="s">
+      <c r="D93" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E93" s="5" t="s">
+      <c r="E93" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F93" s="5" t="s">
+      <c r="F93" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G93" s="9" t="s">
+      <c r="G93" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H93" s="9" t="s">
+      <c r="H93" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I93" s="5" t="n">
+      <c r="I93" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4781,25 +4755,25 @@
       <c r="B94" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C94" s="5" t="s">
+      <c r="C94" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D94" s="5" t="s">
+      <c r="D94" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="E94" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F94" s="5" t="s">
+      <c r="F94" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G94" s="9" t="s">
+      <c r="G94" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H94" s="9" t="s">
+      <c r="H94" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I94" s="5" t="n">
+      <c r="I94" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4810,25 +4784,25 @@
       <c r="B95" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C95" s="5" t="s">
+      <c r="C95" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D95" s="5" t="s">
+      <c r="D95" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E95" s="5" t="s">
+      <c r="E95" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F95" s="5" t="s">
+      <c r="F95" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G95" s="9" t="s">
+      <c r="G95" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H95" s="9" t="s">
+      <c r="H95" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I95" s="5" t="n">
+      <c r="I95" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4839,25 +4813,25 @@
       <c r="B96" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C96" s="5" t="s">
+      <c r="C96" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D96" s="5" t="s">
+      <c r="D96" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E96" s="5" t="s">
+      <c r="E96" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F96" s="5" t="s">
+      <c r="F96" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="G96" s="9" t="s">
+      <c r="G96" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H96" s="9" t="s">
+      <c r="H96" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I96" s="5" t="n">
+      <c r="I96" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4868,25 +4842,25 @@
       <c r="B97" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C97" s="5" t="s">
+      <c r="C97" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D97" s="5" t="s">
+      <c r="D97" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E97" s="5" t="s">
+      <c r="E97" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F97" s="5" t="s">
+      <c r="F97" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G97" s="9" t="s">
+      <c r="G97" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H97" s="5" t="s">
+      <c r="H97" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I97" s="5" t="n">
+      <c r="I97" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -4899,28 +4873,28 @@
       <c r="A100" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B100" s="5" t="s">
+      <c r="B100" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C100" s="5" t="s">
+      <c r="C100" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D100" s="5" t="s">
+      <c r="D100" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E100" s="5" t="s">
+      <c r="E100" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F100" s="5" t="s">
+      <c r="F100" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G100" s="9" t="s">
+      <c r="G100" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H100" s="9" t="s">
+      <c r="H100" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I100" s="5" t="n">
+      <c r="I100" s="2" t="n">
         <v>0.33</v>
       </c>
     </row>
@@ -4928,28 +4902,28 @@
       <c r="A101" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B101" s="5" t="s">
+      <c r="B101" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C101" s="5" t="s">
+      <c r="C101" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D101" s="5" t="s">
+      <c r="D101" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E101" s="5" t="s">
+      <c r="E101" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F101" s="5" t="s">
+      <c r="F101" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G101" s="9" t="s">
+      <c r="G101" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H101" s="9" t="s">
+      <c r="H101" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I101" s="5" t="n">
+      <c r="I101" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4957,90 +4931,89 @@
       <c r="A102" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B102" s="5" t="s">
+      <c r="B102" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C102" s="5" t="s">
+      <c r="C102" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D102" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E102" s="5" t="s">
+      <c r="E102" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F102" s="5" t="s">
+      <c r="F102" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G102" s="9" t="s">
+      <c r="G102" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H102" s="9" t="s">
+      <c r="H102" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I102" s="5" t="n">
+      <c r="I102" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0"/>
-      <c r="C103" s="2"/>
+      <c r="A103" s="7"/>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B104" s="5" t="s">
+      <c r="B104" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C104" s="5" t="s">
+      <c r="C104" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D104" s="5" t="s">
+      <c r="D104" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E104" s="5" t="s">
+      <c r="E104" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F104" s="5" t="s">
+      <c r="F104" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G104" s="9" t="s">
+      <c r="G104" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H104" s="9" t="s">
+      <c r="H104" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I104" s="5" t="n">
-        <v>0.66</v>
+      <c r="I104" s="2" t="n">
+        <v>0.1</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B105" s="5" t="s">
+      <c r="B105" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C105" s="5" t="s">
+      <c r="C105" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D105" s="5" t="s">
+      <c r="D105" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E105" s="5" t="s">
+      <c r="E105" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F105" s="5" t="s">
+      <c r="F105" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G105" s="9" t="s">
+      <c r="G105" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H105" s="9" t="s">
+      <c r="H105" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I105" s="5" t="n">
+      <c r="I105" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -5048,28 +5021,28 @@
       <c r="A106" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B106" s="5" t="s">
+      <c r="B106" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C106" s="5" t="s">
+      <c r="C106" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D106" s="5" t="s">
+      <c r="D106" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E106" s="5" t="s">
+      <c r="E106" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F106" s="5" t="s">
+      <c r="F106" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G106" s="9" t="s">
+      <c r="G106" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H106" s="9" t="s">
+      <c r="H106" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I106" s="5" t="n">
+      <c r="I106" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -5077,28 +5050,28 @@
       <c r="A107" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B107" s="5" t="s">
+      <c r="B107" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C107" s="5" t="s">
+      <c r="C107" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D107" s="5" t="s">
+      <c r="D107" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E107" s="5" t="s">
+      <c r="E107" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F107" s="5" t="s">
+      <c r="F107" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G107" s="9" t="s">
+      <c r="G107" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H107" s="9" t="s">
+      <c r="H107" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I107" s="5" t="n">
+      <c r="I107" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -5106,61 +5079,60 @@
       <c r="A108" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B108" s="5" t="s">
+      <c r="B108" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C108" s="5" t="s">
+      <c r="C108" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D108" s="5" t="s">
+      <c r="D108" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E108" s="5" t="s">
+      <c r="E108" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F108" s="5" t="s">
+      <c r="F108" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G108" s="9" t="s">
+      <c r="G108" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H108" s="9" t="s">
+      <c r="H108" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I108" s="5" t="n">
+      <c r="I108" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="0"/>
-      <c r="C109" s="2"/>
+      <c r="A109" s="7"/>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B110" s="5" t="s">
+      <c r="B110" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C110" s="5" t="s">
+      <c r="C110" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D110" s="5" t="s">
+      <c r="D110" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E110" s="5" t="s">
+      <c r="E110" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F110" s="5" t="s">
+      <c r="F110" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G110" s="9" t="s">
+      <c r="G110" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H110" s="9" t="s">
+      <c r="H110" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I110" s="5" t="n">
+      <c r="I110" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -5168,81 +5140,81 @@
       <c r="A111" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B111" s="5" t="s">
+      <c r="B111" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C111" s="5" t="s">
+      <c r="C111" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D111" s="5" t="s">
+      <c r="D111" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E111" s="5" t="s">
+      <c r="E111" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F111" s="5" t="s">
+      <c r="F111" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G111" s="9" t="s">
+      <c r="G111" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="H111" s="9" t="s">
+      <c r="H111" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I111" s="5" t="n">
+      <c r="I111" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="0"/>
+      <c r="A112" s="7"/>
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0"/>
+      <c r="A113" s="7"/>
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="0"/>
+      <c r="A114" s="7"/>
     </row>
     <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D118" s="0"/>
+      <c r="D118" s="7"/>
     </row>
     <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D119" s="0"/>
+      <c r="D119" s="7"/>
     </row>
     <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D120" s="0"/>
+      <c r="D120" s="7"/>
     </row>
     <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D121" s="0"/>
+      <c r="D121" s="7"/>
     </row>
     <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D122" s="0"/>
+      <c r="D122" s="7"/>
     </row>
     <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D123" s="0"/>
+      <c r="D123" s="7"/>
     </row>
     <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D124" s="0"/>
+      <c r="D124" s="7"/>
     </row>
     <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D125" s="0"/>
+      <c r="D125" s="7"/>
     </row>
     <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D126" s="0"/>
+      <c r="D126" s="7"/>
     </row>
     <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D127" s="0"/>
+      <c r="D127" s="7"/>
     </row>
     <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D128" s="0"/>
+      <c r="D128" s="7"/>
     </row>
     <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D129" s="0"/>
+      <c r="D129" s="7"/>
     </row>
     <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D130" s="0"/>
+      <c r="D130" s="7"/>
     </row>
     <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D131" s="0"/>
+      <c r="D131" s="7"/>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -5282,47 +5254,47 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="15" style="2" width="11.55"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>161</v>
       </c>
     </row>
@@ -5342,10 +5314,10 @@
       <c r="E2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="11" t="n">
+      <c r="F2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="6" t="n">
         <v>3</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -5371,10 +5343,10 @@
       <c r="E3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="11" t="n">
+      <c r="G3" s="6" t="n">
         <v>5</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -5383,7 +5355,7 @@
       <c r="I3" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="L3" s="11"/>
+      <c r="L3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -5401,10 +5373,10 @@
       <c r="E4" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F4" s="11" t="n">
+      <c r="F4" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="G4" s="6" t="n">
         <v>8</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -5413,7 +5385,7 @@
       <c r="I4" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="L4" s="11"/>
+      <c r="L4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -5431,10 +5403,10 @@
       <c r="E5" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="6" t="n">
         <v>12</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -5443,7 +5415,7 @@
       <c r="I5" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="L5" s="11"/>
+      <c r="L5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -5461,10 +5433,10 @@
       <c r="E6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="6" t="n">
         <v>20</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -5473,7 +5445,7 @@
       <c r="I6" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="L6" s="11"/>
+      <c r="L6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5638,10 +5610,10 @@
       <c r="E14" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="6" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="2" t="s">
@@ -5650,8 +5622,7 @@
       <c r="I14" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="J14" s="5"/>
-      <c r="K14" s="9"/>
+      <c r="K14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
@@ -5669,10 +5640,10 @@
       <c r="E15" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="6" t="n">
         <v>7</v>
       </c>
       <c r="H15" s="2" t="s">
@@ -5681,8 +5652,8 @@
       <c r="I15" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
@@ -5700,10 +5671,10 @@
       <c r="E16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="F16" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="6" t="n">
         <v>12</v>
       </c>
       <c r="H16" s="2" t="s">
@@ -5712,8 +5683,7 @@
       <c r="I16" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="9"/>
+      <c r="K16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
@@ -5731,10 +5701,10 @@
       <c r="E17" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F17" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="G17" s="11" t="n">
+      <c r="G17" s="6" t="n">
         <v>19</v>
       </c>
       <c r="H17" s="2" t="s">
@@ -5743,9 +5713,8 @@
       <c r="I17" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="J17" s="5"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="12"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5881,10 +5850,10 @@
       <c r="E24" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F24" s="11" t="n">
+      <c r="F24" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="G24" s="11" t="n">
+      <c r="G24" s="6" t="n">
         <v>10</v>
       </c>
       <c r="H24" s="2" t="s">
@@ -5893,8 +5862,8 @@
       <c r="I24" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="J24" s="11"/>
-      <c r="L24" s="11"/>
+      <c r="J24" s="6"/>
+      <c r="L24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
@@ -5912,10 +5881,10 @@
       <c r="E25" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F25" s="11" t="n">
+      <c r="F25" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="G25" s="11" t="n">
+      <c r="G25" s="6" t="n">
         <v>16</v>
       </c>
       <c r="H25" s="2" t="s">
@@ -5924,8 +5893,8 @@
       <c r="I25" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
@@ -5943,10 +5912,10 @@
       <c r="E26" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="F26" s="11" t="n">
+      <c r="F26" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G26" s="11" t="n">
+      <c r="G26" s="6" t="n">
         <v>20</v>
       </c>
       <c r="H26" s="2" t="s">
@@ -5955,7 +5924,7 @@
       <c r="I26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K26" s="11"/>
+      <c r="K26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
@@ -5973,10 +5942,10 @@
       <c r="E27" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="F27" s="11" t="n">
+      <c r="F27" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="G27" s="11" t="n">
+      <c r="G27" s="6" t="n">
         <v>25</v>
       </c>
       <c r="H27" s="2" t="s">
@@ -5985,8 +5954,8 @@
       <c r="I27" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
@@ -6004,10 +5973,10 @@
       <c r="E28" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F28" s="11" t="n">
+      <c r="F28" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G28" s="11" t="n">
+      <c r="G28" s="6" t="n">
         <v>26</v>
       </c>
       <c r="H28" s="2" t="s">
@@ -6016,9 +5985,9 @@
       <c r="I28" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="0"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6154,10 +6123,10 @@
       <c r="E35" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F35" s="11" t="n">
+      <c r="F35" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G35" s="11" t="n">
+      <c r="G35" s="6" t="n">
         <v>14</v>
       </c>
       <c r="H35" s="2" t="s">
@@ -6166,7 +6135,7 @@
       <c r="I35" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="J35" s="11"/>
+      <c r="J35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
@@ -6184,10 +6153,10 @@
       <c r="E36" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F36" s="11" t="n">
+      <c r="F36" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="G36" s="11" t="n">
+      <c r="G36" s="6" t="n">
         <v>18</v>
       </c>
       <c r="H36" s="2" t="s">
@@ -6196,7 +6165,7 @@
       <c r="I36" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="J36" s="11"/>
+      <c r="J36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
@@ -6214,10 +6183,10 @@
       <c r="E37" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F37" s="11" t="n">
+      <c r="F37" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G37" s="11" t="n">
+      <c r="G37" s="6" t="n">
         <v>26</v>
       </c>
       <c r="H37" s="2" t="s">
@@ -6226,7 +6195,7 @@
       <c r="I37" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="J37" s="11"/>
+      <c r="J37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
@@ -6244,10 +6213,10 @@
       <c r="E38" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="F38" s="11" t="n">
+      <c r="F38" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="G38" s="11" t="n">
+      <c r="G38" s="6" t="n">
         <v>30</v>
       </c>
       <c r="H38" s="2" t="s">
@@ -6256,7 +6225,7 @@
       <c r="I38" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="J38" s="11"/>
+      <c r="J38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6423,50 +6392,50 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>161</v>
       </c>
     </row>
@@ -6533,6 +6502,9 @@
       <c r="J3" s="2" t="n">
         <v>14</v>
       </c>
+      <c r="K3" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -6565,9 +6537,6 @@
       <c r="J4" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="K4" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -6600,9 +6569,6 @@
       <c r="J5" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="K5" s="2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -6699,6 +6665,12 @@
       <c r="J8" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="K8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -6827,6 +6799,12 @@
       <c r="J12" s="2" t="n">
         <v>9</v>
       </c>
+      <c r="K12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
@@ -7179,6 +7157,9 @@
       <c r="J23" s="2" t="n">
         <v>8</v>
       </c>
+      <c r="K23" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
@@ -7626,6 +7607,9 @@
       </c>
       <c r="J37" s="2" t="n">
         <v>15</v>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7805,44 +7789,44 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="7.11"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>161</v>
       </c>
     </row>
@@ -7896,6 +7880,9 @@
       </c>
       <c r="H3" s="2" t="n">
         <v>16</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8157,38 +8144,38 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="4" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>161</v>
       </c>
     </row>
@@ -8263,56 +8250,56 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="2" width="26"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="5" t="s">
         <v>210</v>
       </c>
     </row>
@@ -8857,14 +8844,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>212</v>
       </c>
     </row>
@@ -8907,44 +8894,44 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="10" style="2" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="5" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>223</v>
       </c>
     </row>

</xml_diff>